<commit_message>
feat(0050): 加入 富櫃50 (006201) 平行預測
OTC 也有對應 ETF (006201 元大富櫃50),邏輯同 0050:純市值前 50,被納入 =
被動買盤。OTC 富櫃50 門檻遠小:rank 50 = 362億 / rank 90 = 204億。

- 新增 富櫃50候選A_已體檢:universe ∩ OTC rank 51-90,評分排序
- 新增 富櫃50候選B_blind:OTC rank 51-90 但不在 PICKS
- 新增 OTC前100 分頁:跨板塊對照
- 評分流程與 0050 一致(評等 + 估值 + 拐點 + 距門檻 + 含金量 + 月營收)
</commit_message>
<xml_diff>
--- a/data/台股_0050納入預測.xlsx
+++ b/data/台股_0050納入預測.xlsx
@@ -11,8 +11,10 @@
     <sheet name="候選B_blind_spot" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="universe在TWSE排名" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="TWSE前100" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="OTC轉上市觀察" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="門檻說明" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="富櫃50候選B_blind" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="OTC前100" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="OTC轉上市觀察" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="門檻說明" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3413,7 +3415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3439,302 +3441,929 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>轉上市定位</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>在我們PICKS</t>
+          <t>建議</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5274</t>
+          <t>8932</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>信驊</t>
+          <t>智通*</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6995.4</v>
+        <v>359.8</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>🔥轉上市即進0050(前50)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6223</t>
+          <t>5475</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>旺矽科技</t>
+          <t>德宏工業</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6545.1</v>
+        <v>354.7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>🔥轉上市即進0050(前50)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>53</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8299</t>
+          <t>5425</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>群聯電子</t>
+          <t>台半</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5372.4</v>
+        <v>353.1</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>🔥轉上市即進0050(前50)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>54</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6274</t>
+          <t>3227</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>台燿科技</t>
+          <t>原相科技</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5055.4</v>
+        <v>343.1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>🔥轉上市即進0050(前50)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6488</t>
+          <t>6217</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>環球晶</t>
+          <t>中國探針</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4828.9</v>
+        <v>320</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🔥轉上市即進0050(前50)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5347</t>
+          <t>6023</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>世界先進</t>
+          <t>元大期</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3482.7</v>
+        <v>320</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>⭐轉上市即進51-90</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>57</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3529</t>
+          <t>8086</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>力旺電子</t>
+          <t>宏捷科技</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2378.8</v>
+        <v>313.4</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>⭐轉上市即進51-90</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>8069</t>
+          <t>6640</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>元太</t>
+          <t>均華</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2262.5</v>
+        <v>303.3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>⭐轉上市即進51-90</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>3105</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>穩懋</t>
+          <t>中強光電</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2213</v>
+        <v>299.1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>⭐轉上市即進51-90</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3293</t>
+          <t>5439</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>鈊象電子</t>
+          <t>高技企業</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2141.7</v>
+        <v>298.9</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>⭐轉上市即進51-90</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3081</t>
+          <t>5351</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>聯亞</t>
+          <t>鈺創科技</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2114</v>
+        <v>298.9</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>⭐轉上市即進51-90</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>6147</t>
+          <t>8064</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>頎邦科技</t>
+          <t>東捷科技</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1921</v>
+        <v>288.3</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>⭐轉上市即進51-90</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>63</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>4123</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>晟德</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>286.8</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>64</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>6613</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>朋億*</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>286.3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>65</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>先進光</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>274.2</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>66</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>6138</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>茂達電子</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>273</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>67</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>6561</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>是方</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>265.1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>68</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>6739</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>竹陞科技</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>262</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>69</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>8027</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>鈦昇</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>260.7</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>70</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>6903</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>巨漢</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>254</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>71</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>3265</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>台星科</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>247.3</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>72</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>8155</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>博智</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>239.3</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>73</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>3675</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>德微</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>236.4</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>74</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>4743</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>合一</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>233.5</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>75</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>8042</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>金山電子</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>230.6</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>76</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>6664</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>群翊</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>229</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>77</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>6291</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>沛亨半導</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>228.1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>78</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>5864</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>致和證</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>226.6</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>79</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>8096</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>擎亞</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>224.8</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>80</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>7805</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>威聯通</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>224.6</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>81</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>3587</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>閎康科技</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>217.4</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>82</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>5009</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>榮剛材料</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>216.9</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>83</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>6188</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>廣明光電</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>216.3</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>84</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>4971</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>IET-KY</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>215.9</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>85</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>3693</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>營邦</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>213.2</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>86</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>4506</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>崇友實業</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>210.6</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>87</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>6803</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>崑鼎</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>208.6</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>88</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>4728</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>雙美</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>205.1</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>89</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>6643</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>M31</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>205</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>90</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>3526</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>凡甲科技</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>203.5</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>加入 PICKS 抓體檢</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3747,6 +4376,2481 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>代號</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>名稱</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>收盤</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>市值億</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5274</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>信驊</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>18505</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6995.4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>6223</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>旺矽科技</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6680</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6545.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>8299</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>群聯電子</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2430</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5372.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>6274</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>台燿科技</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1735</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5055.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>6488</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>環球晶</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1010</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4828.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5347</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>世界先進</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>186.5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3482.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>3529</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>力旺電子</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3185</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2378.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8069</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>元太</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>196</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2262.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>3105</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>穩懋</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>522</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2213</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>3293</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>鈊象電子</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>760</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2141.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2285</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2114</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>頎邦科技</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>258</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1921</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>5289</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>宜鼎</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1885</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1816.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>8358</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>金居開發</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>657</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1659.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>5536</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>聖暉*</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1260</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1563.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>3260</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>威剛科技</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>412</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1357.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>6510</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>精測</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3665</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1205.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>6187</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>萬潤</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1170</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1148.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>3264</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>欣銓科技</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>233.5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1144.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>5483</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>中美晶</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>173.5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1112.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>3131</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>弘塑科技</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>3495</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1037.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>3324</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>雙鴻科技</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1025</v>
+      </c>
+      <c r="E23" t="n">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>7734</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>印能科技</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3390</v>
+      </c>
+      <c r="E24" t="n">
+        <v>949.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>3491</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>昇達科技</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1355</v>
+      </c>
+      <c r="E25" t="n">
+        <v>932.3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>7828</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>創新服務</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2240</v>
+      </c>
+      <c r="E26" t="n">
+        <v>907.1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1785</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>光洋科技</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>149.5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>6548</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>長科*</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>92.7</v>
+      </c>
+      <c r="E28" t="n">
+        <v>881.1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>4749</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>新應材</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>917</v>
+      </c>
+      <c r="E29" t="n">
+        <v>868.7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3374</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>精材</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>303.5</v>
+      </c>
+      <c r="E30" t="n">
+        <v>823.6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3363</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>上詮</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>685</v>
+      </c>
+      <c r="E31" t="n">
+        <v>778.4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>6121</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>新普科技</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>417</v>
+      </c>
+      <c r="E32" t="n">
+        <v>771.3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>4979</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>華星光</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>525</v>
+      </c>
+      <c r="E33" t="n">
+        <v>747.4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>5904</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>寶雅國際</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>666</v>
+      </c>
+      <c r="E34" t="n">
+        <v>708.9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>3163</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>波若威</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>868</v>
+      </c>
+      <c r="E35" t="n">
+        <v>699.1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>6182</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>合晶科技</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>114.5</v>
+      </c>
+      <c r="E36" t="n">
+        <v>679.7</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>3211</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>順達科技</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>427.5</v>
+      </c>
+      <c r="E37" t="n">
+        <v>660.1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>4991</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>環宇-KY</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>536</v>
+      </c>
+      <c r="E38" t="n">
+        <v>648.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1815</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>富喬</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="E39" t="n">
+        <v>588.4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>4966</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>譜瑞-KY</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>661</v>
+      </c>
+      <c r="E40" t="n">
+        <v>521.9</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>6290</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>良維科技</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>306</v>
+      </c>
+      <c r="E41" t="n">
+        <v>518.7</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>3680</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>家登</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>537</v>
+      </c>
+      <c r="E42" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>6173</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>信昌電陶</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>285</v>
+      </c>
+      <c r="E43" t="n">
+        <v>490.2</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>6683</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>雍智科技</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>1765</v>
+      </c>
+      <c r="E44" t="n">
+        <v>486.4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>6584</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>南俊國際</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>649</v>
+      </c>
+      <c r="E45" t="n">
+        <v>460.3</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>5903</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>全家</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>188.5</v>
+      </c>
+      <c r="E46" t="n">
+        <v>420.8</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>4772</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>台特化</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>275</v>
+      </c>
+      <c r="E47" t="n">
+        <v>406.1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>3707</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>漢磊</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="E48" t="n">
+        <v>398.6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>7751</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>竑騰</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1475</v>
+      </c>
+      <c r="E49" t="n">
+        <v>396.6</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>8415</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>大國鋼</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>35.25</v>
+      </c>
+      <c r="E50" t="n">
+        <v>363.6</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>3357</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>臺慶科</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>315</v>
+      </c>
+      <c r="E51" t="n">
+        <v>362.1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>8932</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>智通*</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="E52" t="n">
+        <v>359.8</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>5475</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>德宏工業</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>279</v>
+      </c>
+      <c r="E53" t="n">
+        <v>354.7</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>5425</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>台半</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>134</v>
+      </c>
+      <c r="E54" t="n">
+        <v>353.1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>3227</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>原相科技</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>228</v>
+      </c>
+      <c r="E55" t="n">
+        <v>343.1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>6217</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>中國探針</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>273</v>
+      </c>
+      <c r="E56" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>6023</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>元大期</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>100</v>
+      </c>
+      <c r="E57" t="n">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>8086</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>宏捷科技</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>159.5</v>
+      </c>
+      <c r="E58" t="n">
+        <v>313.4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>6640</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>均華</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>1050</v>
+      </c>
+      <c r="E59" t="n">
+        <v>303.3</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>5371</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>中強光電</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="E60" t="n">
+        <v>299.1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>5439</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>高技企業</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>321.5</v>
+      </c>
+      <c r="E61" t="n">
+        <v>298.9</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>5351</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>鈺創科技</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>91</v>
+      </c>
+      <c r="E62" t="n">
+        <v>298.9</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>8064</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>東捷科技</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>156</v>
+      </c>
+      <c r="E63" t="n">
+        <v>288.3</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>4123</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>晟德</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>37.3</v>
+      </c>
+      <c r="E64" t="n">
+        <v>286.8</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>6613</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>朋億*</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>368</v>
+      </c>
+      <c r="E65" t="n">
+        <v>286.3</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>先進光</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>186</v>
+      </c>
+      <c r="E66" t="n">
+        <v>274.2</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>6138</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>茂達電子</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>361</v>
+      </c>
+      <c r="E67" t="n">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>6561</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>是方</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>340</v>
+      </c>
+      <c r="E68" t="n">
+        <v>265.1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>6739</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>竹陞科技</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>1120</v>
+      </c>
+      <c r="E69" t="n">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>8027</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>鈦昇</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>237</v>
+      </c>
+      <c r="E70" t="n">
+        <v>260.7</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>6903</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>巨漢</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>381</v>
+      </c>
+      <c r="E71" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>3265</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>台星科</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>181.5</v>
+      </c>
+      <c r="E72" t="n">
+        <v>247.3</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>8155</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>博智</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>388.5</v>
+      </c>
+      <c r="E73" t="n">
+        <v>239.3</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>3675</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>德微</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>445.5</v>
+      </c>
+      <c r="E74" t="n">
+        <v>236.4</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>4743</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>合一</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="E75" t="n">
+        <v>233.5</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>8042</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>金山電子</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>177.5</v>
+      </c>
+      <c r="E76" t="n">
+        <v>230.6</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>6664</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>群翊</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>376.5</v>
+      </c>
+      <c r="E77" t="n">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>6291</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>沛亨半導</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>543</v>
+      </c>
+      <c r="E78" t="n">
+        <v>228.1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>5864</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>致和證</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>49.85</v>
+      </c>
+      <c r="E79" t="n">
+        <v>226.6</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>8096</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>擎亞</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>150.5</v>
+      </c>
+      <c r="E80" t="n">
+        <v>224.8</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>7805</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>威聯通</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>678</v>
+      </c>
+      <c r="E81" t="n">
+        <v>224.6</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>3587</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>閎康科技</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>305.5</v>
+      </c>
+      <c r="E82" t="n">
+        <v>217.4</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>5009</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>榮剛材料</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>36</v>
+      </c>
+      <c r="E83" t="n">
+        <v>216.9</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>6188</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>廣明光電</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="E84" t="n">
+        <v>216.3</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>4971</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>IET-KY</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>540</v>
+      </c>
+      <c r="E85" t="n">
+        <v>215.9</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>3693</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>營邦</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>496</v>
+      </c>
+      <c r="E86" t="n">
+        <v>213.2</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>4506</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>崇友實業</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>119</v>
+      </c>
+      <c r="E87" t="n">
+        <v>210.6</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>6803</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>崑鼎</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>286.5</v>
+      </c>
+      <c r="E88" t="n">
+        <v>208.6</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>4728</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>雙美</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>376.5</v>
+      </c>
+      <c r="E89" t="n">
+        <v>205.1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>6643</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>M31</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>490.5</v>
+      </c>
+      <c r="E90" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>3526</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>凡甲科技</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>309</v>
+      </c>
+      <c r="E91" t="n">
+        <v>203.5</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>5530</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>龍巖</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="E92" t="n">
+        <v>203.1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>8255</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>朋程</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>199.5</v>
+      </c>
+      <c r="E93" t="n">
+        <v>203.1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>6016</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>康和證券</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>29.15</v>
+      </c>
+      <c r="E94" t="n">
+        <v>200.1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>6146</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>耕興</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>191.5</v>
+      </c>
+      <c r="E95" t="n">
+        <v>195.1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>5340</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>建榮工業</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>96</v>
+      </c>
+      <c r="E96" t="n">
+        <v>187.1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>3624</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>光頡科技</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>159</v>
+      </c>
+      <c r="E97" t="n">
+        <v>186.6</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>4105</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>東洋藥品</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>73.90000000000001</v>
+      </c>
+      <c r="E98" t="n">
+        <v>183.8</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>5386</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>青雲國際</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>502</v>
+      </c>
+      <c r="E99" t="n">
+        <v>181.1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>4768</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>晶呈科技</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>374</v>
+      </c>
+      <c r="E100" t="n">
+        <v>177.6</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>5314</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>世紀*</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="E101" t="n">
+        <v>176.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>OTC排名</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>代號</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>名稱</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>市值億</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>轉上市定位</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>在我們PICKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5274</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>信驊</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6995.4</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>🔥轉上市即進0050(前50)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>6223</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>旺矽科技</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6545.1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>🔥轉上市即進0050(前50)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>8299</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>群聯電子</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5372.4</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>🔥轉上市即進0050(前50)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>6274</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>台燿科技</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5055.4</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>🔥轉上市即進0050(前50)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>6488</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>環球晶</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4828.9</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>🔥轉上市即進0050(前50)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>5347</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>世界先進</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3482.7</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>⭐轉上市即進51-90</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>3529</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>力旺電子</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2378.8</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>⭐轉上市即進51-90</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8069</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>元太</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2262.5</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>⭐轉上市即進51-90</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>3105</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>穩懋</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2213</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>⭐轉上市即進51-90</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>3293</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>鈊象電子</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2141.7</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>⭐轉上市即進51-90</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2114</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>⭐轉上市即進51-90</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>頎邦科技</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1921</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>⭐轉上市即進51-90</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
data: 正式產出(247檔,含 Forward PE/PEG 全鏈)20260623
</commit_message>
<xml_diff>
--- a/data/台股_0050納入預測.xlsx
+++ b/data/台股_0050納入預測.xlsx
@@ -590,7 +590,9 @@
       <c r="O2" t="n">
         <v>1.13</v>
       </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="P2" t="n">
+        <v>2974.9</v>
+      </c>
       <c r="Q2" t="n">
         <v>27.5</v>
       </c>
@@ -662,7 +664,9 @@
       <c r="O3" t="n">
         <v>2.64</v>
       </c>
-      <c r="P3" t="inlineStr"/>
+      <c r="P3" t="n">
+        <v>2439.5</v>
+      </c>
       <c r="Q3" t="n">
         <v>23.77</v>
       </c>
@@ -798,7 +802,9 @@
       <c r="O5" t="n">
         <v>1</v>
       </c>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="n">
+        <v>4027</v>
+      </c>
       <c r="Q5" t="n">
         <v>65.19</v>
       </c>
@@ -864,7 +870,9 @@
       <c r="O6" t="n">
         <v>1.62</v>
       </c>
-      <c r="P6" t="inlineStr"/>
+      <c r="P6" t="n">
+        <v>3092.8</v>
+      </c>
       <c r="Q6" t="n">
         <v>45.77</v>
       </c>
@@ -1078,7 +1086,9 @@
       <c r="O9" t="n">
         <v>0.63</v>
       </c>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="n">
+        <v>3409.2</v>
+      </c>
       <c r="Q9" t="n">
         <v>192.04</v>
       </c>
@@ -1154,7 +1164,9 @@
       <c r="O10" t="n">
         <v>2.4</v>
       </c>
-      <c r="P10" t="inlineStr"/>
+      <c r="P10" t="n">
+        <v>3895.6</v>
+      </c>
       <c r="Q10" t="n">
         <v>27.34</v>
       </c>
@@ -1216,7 +1228,9 @@
       <c r="O11" t="n">
         <v>-0.2</v>
       </c>
-      <c r="P11" t="inlineStr"/>
+      <c r="P11" t="n">
+        <v>2855.6</v>
+      </c>
       <c r="Q11" t="n">
         <v>15.52</v>
       </c>
@@ -1292,7 +1306,9 @@
       <c r="O12" t="n">
         <v>1.12</v>
       </c>
-      <c r="P12" t="inlineStr"/>
+      <c r="P12" t="n">
+        <v>2625</v>
+      </c>
       <c r="Q12" t="n">
         <v>57.11</v>
       </c>
@@ -1362,7 +1378,9 @@
       <c r="O13" t="n">
         <v>2.01</v>
       </c>
-      <c r="P13" t="inlineStr"/>
+      <c r="P13" t="n">
+        <v>2778.5</v>
+      </c>
       <c r="Q13" t="n">
         <v>43.57</v>
       </c>
@@ -1498,7 +1516,9 @@
       <c r="O15" t="n">
         <v>-1.14</v>
       </c>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="n">
+        <v>2304.4</v>
+      </c>
       <c r="Q15" t="n">
         <v>16.07</v>
       </c>
@@ -1638,7 +1658,9 @@
       <c r="O17" t="n">
         <v>9.07</v>
       </c>
-      <c r="P17" t="inlineStr"/>
+      <c r="P17" t="n">
+        <v>2227.6</v>
+      </c>
       <c r="Q17" t="n">
         <v>589.23</v>
       </c>
@@ -1704,7 +1726,9 @@
       <c r="O18" t="n">
         <v>-11.39</v>
       </c>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="n">
+        <v>546.8</v>
+      </c>
       <c r="Q18" t="n">
         <v>18.01</v>
       </c>
@@ -1838,7 +1862,9 @@
       <c r="O20" t="n">
         <v>-0.89</v>
       </c>
-      <c r="P20" t="inlineStr"/>
+      <c r="P20" t="n">
+        <v>1889</v>
+      </c>
       <c r="Q20" t="n">
         <v>14.17</v>
       </c>
@@ -2040,7 +2066,9 @@
       <c r="O23" t="n">
         <v>0.7</v>
       </c>
-      <c r="P23" t="inlineStr"/>
+      <c r="P23" t="n">
+        <v>1715.8</v>
+      </c>
       <c r="Q23" t="n">
         <v>30.21</v>
       </c>

</xml_diff>

<commit_message>
data: 0050 納入預測 20260624
</commit_message>
<xml_diff>
--- a/data/台股_0050納入預測.xlsx
+++ b/data/台股_0050納入預測.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="候選A_已體檢" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="候選B_blind_spot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="universe在TWSE排名" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TWSE前100" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="富櫃50候選A_已體檢" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="富櫃50候選B_blind" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="OTC前100" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="OTC轉上市觀察" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="門檻說明" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="候選A_已體檢" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="候選B_blind_spot" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="universe在TWSE排名" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TWSE前100" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="富櫃50候選A_已體檢" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="富櫃50候選B_blind" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OTC前100" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OTC轉上市觀察" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="門檻說明" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,13 +25,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,116 +433,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TWSE排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>大盤比重%</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>納入潛力分</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>評等</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>品質總分</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>估值</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>未來估值</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>PEG</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>ForwardPE</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>成長率g%</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>改善訊號數</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>分級</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>含金量</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>市值(億)</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>PER(自算)</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>PE位階%</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>PBR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>殖利率%</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>最新月營收年增%</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>循環股</t>
         </is>
@@ -538,97 +530,87 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3044</t>
+          <t>6446</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>健鼎</t>
+          <t>藥華藥</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.1883</v>
+        <v>0.2429</v>
       </c>
       <c r="E2" t="n">
-        <v>105</v>
+        <v>85</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>🟢成長未反映</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>0.92</v>
-      </c>
+          <t>🟠偏貴</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
-        <v>21.2</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>29.8</v>
+        <v>4027</v>
       </c>
       <c r="M2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
+        <v>65.19</v>
+      </c>
+      <c r="N2" t="n">
+        <v>59</v>
+      </c>
       <c r="O2" t="n">
-        <v>1.13</v>
+        <v>11.44</v>
       </c>
       <c r="P2" t="n">
-        <v>2974.9</v>
+        <v>0.25</v>
       </c>
       <c r="Q2" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="R2" t="n">
-        <v>100</v>
-      </c>
-      <c r="S2" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="T2" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="U2" t="n">
-        <v>46.6</v>
-      </c>
-      <c r="V2" t="inlineStr"/>
+        <v>108.5</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>⚠️循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2404</t>
+          <t>3044</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>漢唐</t>
+          <t>健鼎</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.1514</v>
+        <v>0.1883</v>
       </c>
       <c r="E3" t="n">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -636,73 +618,59 @@
         </is>
       </c>
       <c r="G3" t="n">
+        <v>90</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2974.9</v>
+      </c>
+      <c r="M3" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="N3" t="n">
         <v>100</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>🔴過熱</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>🟢成長未反映</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="K3" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="L3" t="n">
-        <v>39.2</v>
-      </c>
-      <c r="M3" t="n">
-        <v>3</v>
-      </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>2.64</v>
+        <v>5.1</v>
       </c>
       <c r="P3" t="n">
-        <v>2439.5</v>
+        <v>2.24</v>
       </c>
       <c r="Q3" t="n">
-        <v>23.77</v>
-      </c>
-      <c r="R3" t="n">
-        <v>96</v>
-      </c>
-      <c r="S3" t="n">
-        <v>16.81</v>
-      </c>
-      <c r="T3" t="n">
-        <v>3.13</v>
-      </c>
-      <c r="U3" t="n">
-        <v>85</v>
-      </c>
-      <c r="V3" t="inlineStr"/>
+        <v>46.6</v>
+      </c>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>84</v>
+        <v>55</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6139</t>
+          <t>2313</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>亞翔</t>
+          <t>華通</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.127</v>
+        <v>0.2331</v>
       </c>
       <c r="E4" t="n">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -710,138 +678,120 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>🟢成長未反映</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>0.4</v>
-      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
-        <v>14.2</v>
+        <v>1.62</v>
       </c>
       <c r="L4" t="n">
-        <v>54.3</v>
+        <v>3092.8</v>
       </c>
       <c r="M4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N4" t="inlineStr"/>
+        <v>45.77</v>
+      </c>
+      <c r="N4" t="n">
+        <v>97</v>
+      </c>
       <c r="O4" t="n">
-        <v>1.56</v>
+        <v>6.6</v>
       </c>
       <c r="P4" t="n">
-        <v>1863.4</v>
+        <v>1.08</v>
       </c>
       <c r="Q4" t="n">
-        <v>21.89</v>
-      </c>
-      <c r="R4" t="n">
-        <v>74</v>
-      </c>
-      <c r="S4" t="n">
-        <v>8.51</v>
-      </c>
-      <c r="T4" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="U4" t="n">
-        <v>103.3</v>
-      </c>
-      <c r="V4" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>⚠️循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6446</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>藥華藥</t>
+          <t>漢唐</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.2429</v>
+        <v>0.1514</v>
       </c>
       <c r="E5" t="n">
+        <v>78</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2439.5</v>
+      </c>
+      <c r="M5" t="n">
+        <v>23.77</v>
+      </c>
+      <c r="N5" t="n">
+        <v>96</v>
+      </c>
+      <c r="O5" t="n">
+        <v>16.81</v>
+      </c>
+      <c r="P5" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="Q5" t="n">
         <v>85</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>66</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>🟠偏貴</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="n">
-        <v>2</v>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" t="n">
-        <v>4027</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>65.19</v>
-      </c>
-      <c r="R5" t="n">
-        <v>59</v>
-      </c>
-      <c r="S5" t="n">
-        <v>11.44</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="U5" t="n">
-        <v>108.5</v>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>⚠️循環(看PBR)</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2313</t>
+          <t>6139</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>華通</t>
+          <t>亞翔</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.2331</v>
+        <v>0.127</v>
       </c>
       <c r="E6" t="n">
         <v>78</v>
@@ -852,67 +802,59 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1863.4</v>
+      </c>
       <c r="M6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="inlineStr"/>
+        <v>21.89</v>
+      </c>
+      <c r="N6" t="n">
+        <v>74</v>
+      </c>
       <c r="O6" t="n">
-        <v>1.62</v>
+        <v>8.51</v>
       </c>
       <c r="P6" t="n">
-        <v>3092.8</v>
+        <v>2.91</v>
       </c>
       <c r="Q6" t="n">
-        <v>45.77</v>
-      </c>
-      <c r="R6" t="n">
-        <v>97</v>
-      </c>
-      <c r="S6" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="T6" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="U6" t="n">
-        <v>13</v>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>⚠️循環(看PBR)</t>
-        </is>
-      </c>
+        <v>103.3</v>
+      </c>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2356</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>英業達</t>
+          <t>亞德客-KY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.1732</v>
+        <v>0.1925</v>
       </c>
       <c r="E7" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -924,211 +866,179 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>🟡未來合理</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>1.35</v>
-      </c>
+          <t>🟠偏貴</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>21.3</v>
+        <v>0.98</v>
       </c>
       <c r="L7" t="n">
-        <v>18.7</v>
+        <v>2750</v>
       </c>
       <c r="M7" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" t="inlineStr"/>
+        <v>30.1</v>
+      </c>
+      <c r="N7" t="n">
+        <v>66</v>
+      </c>
       <c r="O7" t="n">
-        <v>1.09</v>
+        <v>5.41</v>
       </c>
       <c r="P7" t="n">
-        <v>2371.3</v>
+        <v>2.12</v>
       </c>
       <c r="Q7" t="n">
-        <v>25.23</v>
-      </c>
-      <c r="R7" t="n">
-        <v>72</v>
-      </c>
-      <c r="S7" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="T7" t="n">
-        <v>3.03</v>
-      </c>
-      <c r="U7" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="V7" t="inlineStr"/>
+        <v>40.4</v>
+      </c>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>6515</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>亞德客-KY</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.1925</v>
+        <v>0.2147</v>
       </c>
       <c r="E8" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>🟠未來偏貴</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>3.06</v>
-      </c>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>27.4</v>
+        <v>0.63</v>
       </c>
       <c r="L8" t="n">
-        <v>9.800000000000001</v>
+        <v>3409.2</v>
       </c>
       <c r="M8" t="n">
-        <v>4</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
+        <v>192.04</v>
+      </c>
+      <c r="N8" t="n">
+        <v>98</v>
+      </c>
       <c r="O8" t="n">
-        <v>0.98</v>
+        <v>52.47</v>
       </c>
       <c r="P8" t="n">
-        <v>2750</v>
+        <v>0.53</v>
       </c>
       <c r="Q8" t="n">
-        <v>30.1</v>
-      </c>
-      <c r="R8" t="n">
-        <v>66</v>
-      </c>
-      <c r="S8" t="n">
-        <v>5.41</v>
-      </c>
-      <c r="T8" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="U8" t="n">
-        <v>40.4</v>
-      </c>
-      <c r="V8" t="inlineStr"/>
+        <v>119.8</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>⚠️循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6515</t>
+          <t>4904</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>遠傳</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.2147</v>
+        <v>0.2285</v>
       </c>
       <c r="E9" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="K9" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3895.6</v>
+      </c>
       <c r="M9" t="n">
-        <v>2</v>
-      </c>
-      <c r="N9" t="inlineStr"/>
+        <v>27.34</v>
+      </c>
+      <c r="N9" t="n">
+        <v>95</v>
+      </c>
       <c r="O9" t="n">
-        <v>0.63</v>
+        <v>4.06</v>
       </c>
       <c r="P9" t="n">
-        <v>3409.2</v>
+        <v>3.53</v>
       </c>
       <c r="Q9" t="n">
-        <v>192.04</v>
-      </c>
-      <c r="R9" t="n">
-        <v>98</v>
-      </c>
-      <c r="S9" t="n">
-        <v>52.47</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="U9" t="n">
-        <v>119.8</v>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>⚠️循環(看PBR)</t>
-        </is>
-      </c>
+        <v>13.7</v>
+      </c>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4904</t>
+          <t>2356</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>遠傳</t>
+          <t>英業達</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.2285</v>
+        <v>0.1732</v>
       </c>
       <c r="E10" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1136,53 +1046,39 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>🟠未來偏貴</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>4.94</v>
-      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>25.9</v>
+        <v>1.09</v>
       </c>
       <c r="L10" t="n">
-        <v>5.5</v>
+        <v>2371.3</v>
       </c>
       <c r="M10" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" t="inlineStr"/>
+        <v>25.23</v>
+      </c>
+      <c r="N10" t="n">
+        <v>72</v>
+      </c>
       <c r="O10" t="n">
-        <v>2.4</v>
+        <v>3.23</v>
       </c>
       <c r="P10" t="n">
-        <v>3895.6</v>
+        <v>3.03</v>
       </c>
       <c r="Q10" t="n">
-        <v>27.34</v>
-      </c>
-      <c r="R10" t="n">
-        <v>95</v>
-      </c>
-      <c r="S10" t="n">
-        <v>4.06</v>
-      </c>
-      <c r="T10" t="n">
-        <v>3.53</v>
-      </c>
-      <c r="U10" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="V10" t="inlineStr"/>
+        <v>35.3</v>
+      </c>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1217,36 +1113,32 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>3</v>
+      </c>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2855.6</v>
+      </c>
       <c r="M11" t="n">
-        <v>3</v>
-      </c>
-      <c r="N11" t="inlineStr"/>
+        <v>15.52</v>
+      </c>
+      <c r="N11" t="n">
+        <v>68</v>
+      </c>
       <c r="O11" t="n">
-        <v>-0.2</v>
+        <v>2.53</v>
       </c>
       <c r="P11" t="n">
-        <v>2855.6</v>
+        <v>3.47</v>
       </c>
       <c r="Q11" t="n">
-        <v>15.52</v>
-      </c>
-      <c r="R11" t="n">
-        <v>68</v>
-      </c>
-      <c r="S11" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="T11" t="n">
-        <v>3.47</v>
-      </c>
-      <c r="U11" t="n">
         <v>152.7</v>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -1285,46 +1177,32 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>🔴未來過熱</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>2.83</v>
-      </c>
+      <c r="I12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>47.5</v>
+        <v>1.12</v>
       </c>
       <c r="L12" t="n">
-        <v>20.2</v>
+        <v>2625</v>
       </c>
       <c r="M12" t="n">
-        <v>2</v>
-      </c>
-      <c r="N12" t="inlineStr"/>
+        <v>57.11</v>
+      </c>
+      <c r="N12" t="n">
+        <v>84</v>
+      </c>
       <c r="O12" t="n">
-        <v>1.12</v>
+        <v>31.86</v>
       </c>
       <c r="P12" t="n">
-        <v>2625</v>
+        <v>1.44</v>
       </c>
       <c r="Q12" t="n">
-        <v>57.11</v>
-      </c>
-      <c r="R12" t="n">
-        <v>84</v>
-      </c>
-      <c r="S12" t="n">
-        <v>31.86</v>
-      </c>
-      <c r="T12" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="U12" t="n">
         <v>-9.300000000000001</v>
       </c>
-      <c r="V12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1359,44 +1237,32 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>🔴未來過熱</t>
-        </is>
+      <c r="I13" t="n">
+        <v>2</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>52.2</v>
+        <v>2.01</v>
       </c>
       <c r="L13" t="n">
-        <v>-16.5</v>
+        <v>2778.5</v>
       </c>
       <c r="M13" t="n">
-        <v>2</v>
-      </c>
-      <c r="N13" t="inlineStr"/>
+        <v>43.57</v>
+      </c>
+      <c r="N13" t="n">
+        <v>100</v>
+      </c>
       <c r="O13" t="n">
-        <v>2.01</v>
+        <v>4.63</v>
       </c>
       <c r="P13" t="n">
-        <v>2778.5</v>
+        <v>1.23</v>
       </c>
       <c r="Q13" t="n">
-        <v>43.57</v>
-      </c>
-      <c r="R13" t="n">
-        <v>100</v>
-      </c>
-      <c r="S13" t="n">
-        <v>4.63</v>
-      </c>
-      <c r="T13" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="U13" t="n">
         <v>30.2</v>
       </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1431,46 +1297,32 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>🟠未來偏貴</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>1.76</v>
-      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="n">
-        <v>26.6</v>
+        <v>0.89</v>
       </c>
       <c r="L14" t="n">
-        <v>17.8</v>
+        <v>2515.2</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="inlineStr"/>
+        <v>31.35</v>
+      </c>
+      <c r="N14" t="n">
+        <v>96</v>
+      </c>
       <c r="O14" t="n">
-        <v>0.89</v>
+        <v>5.98</v>
       </c>
       <c r="P14" t="n">
-        <v>2515.2</v>
+        <v>1.57</v>
       </c>
       <c r="Q14" t="n">
-        <v>31.35</v>
-      </c>
-      <c r="R14" t="n">
-        <v>96</v>
-      </c>
-      <c r="S14" t="n">
-        <v>5.98</v>
-      </c>
-      <c r="T14" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="U14" t="n">
         <v>9</v>
       </c>
-      <c r="V14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1505,36 +1357,32 @@
           <t>🟢便宜</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
       <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2304.4</v>
+      </c>
       <c r="M15" t="n">
-        <v>3</v>
-      </c>
-      <c r="N15" t="inlineStr"/>
+        <v>16.07</v>
+      </c>
+      <c r="N15" t="n">
+        <v>52</v>
+      </c>
       <c r="O15" t="n">
-        <v>-1.14</v>
+        <v>1.43</v>
       </c>
       <c r="P15" t="n">
-        <v>2304.4</v>
+        <v>4.99</v>
       </c>
       <c r="Q15" t="n">
-        <v>16.07</v>
-      </c>
-      <c r="R15" t="n">
-        <v>52</v>
-      </c>
-      <c r="S15" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="T15" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="U15" t="n">
         <v>5</v>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -1573,46 +1421,32 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>🔴未來過熱</t>
-        </is>
-      </c>
-      <c r="J16" t="n">
-        <v>2.73</v>
-      </c>
+      <c r="I16" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
-        <v>51.7</v>
+        <v>0.26</v>
       </c>
       <c r="L16" t="n">
-        <v>23.4</v>
+        <v>3567.1</v>
       </c>
       <c r="M16" t="n">
-        <v>2</v>
-      </c>
-      <c r="N16" t="inlineStr"/>
+        <v>63.77</v>
+      </c>
+      <c r="N16" t="n">
+        <v>82</v>
+      </c>
       <c r="O16" t="n">
-        <v>0.26</v>
+        <v>8.27</v>
       </c>
       <c r="P16" t="n">
-        <v>3567.1</v>
+        <v>0.78</v>
       </c>
       <c r="Q16" t="n">
-        <v>63.77</v>
-      </c>
-      <c r="R16" t="n">
-        <v>82</v>
-      </c>
-      <c r="S16" t="n">
-        <v>8.27</v>
-      </c>
-      <c r="T16" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="U16" t="n">
         <v>-33.5</v>
       </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1647,36 +1481,32 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>2</v>
+      </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2227.6</v>
+      </c>
       <c r="M17" t="n">
-        <v>2</v>
-      </c>
-      <c r="N17" t="inlineStr"/>
+        <v>589.23</v>
+      </c>
+      <c r="N17" t="n">
+        <v>96</v>
+      </c>
       <c r="O17" t="n">
-        <v>9.07</v>
+        <v>4.48</v>
       </c>
       <c r="P17" t="n">
-        <v>2227.6</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>589.23</v>
-      </c>
-      <c r="R17" t="n">
-        <v>96</v>
-      </c>
-      <c r="S17" t="n">
-        <v>4.48</v>
-      </c>
-      <c r="T17" t="n">
-        <v>0</v>
-      </c>
-      <c r="U17" t="n">
         <v>17.7</v>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -1715,36 +1545,32 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+      <c r="K18" t="n">
+        <v>-11.39</v>
+      </c>
+      <c r="L18" t="n">
+        <v>546.8</v>
+      </c>
       <c r="M18" t="n">
-        <v>2</v>
-      </c>
-      <c r="N18" t="inlineStr"/>
+        <v>18.01</v>
+      </c>
+      <c r="N18" t="n">
+        <v>91</v>
+      </c>
       <c r="O18" t="n">
-        <v>-11.39</v>
+        <v>7.25</v>
       </c>
       <c r="P18" t="n">
-        <v>546.8</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>18.01</v>
-      </c>
-      <c r="R18" t="n">
-        <v>91</v>
-      </c>
-      <c r="S18" t="n">
-        <v>7.25</v>
-      </c>
-      <c r="T18" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" t="n">
         <v>175.8</v>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -1783,36 +1609,32 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="L19" t="n">
+        <v>3310.3</v>
+      </c>
       <c r="M19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N19" t="inlineStr"/>
+        <v>22.29</v>
+      </c>
+      <c r="N19" t="n">
+        <v>97</v>
+      </c>
       <c r="O19" t="n">
-        <v>1.01</v>
+        <v>4.6</v>
       </c>
       <c r="P19" t="n">
-        <v>3310.3</v>
+        <v>4.23</v>
       </c>
       <c r="Q19" t="n">
-        <v>22.29</v>
-      </c>
-      <c r="R19" t="n">
-        <v>97</v>
-      </c>
-      <c r="S19" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="T19" t="n">
-        <v>4.23</v>
-      </c>
-      <c r="U19" t="n">
         <v>9.4</v>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -1851,36 +1673,32 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>3</v>
+      </c>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="L20" t="n">
+        <v>1889</v>
+      </c>
       <c r="M20" t="n">
-        <v>3</v>
-      </c>
-      <c r="N20" t="inlineStr"/>
+        <v>14.17</v>
+      </c>
+      <c r="N20" t="n">
+        <v>62</v>
+      </c>
       <c r="O20" t="n">
-        <v>-0.89</v>
+        <v>2.1</v>
       </c>
       <c r="P20" t="n">
-        <v>1889</v>
+        <v>3.38</v>
       </c>
       <c r="Q20" t="n">
-        <v>14.17</v>
-      </c>
-      <c r="R20" t="n">
-        <v>62</v>
-      </c>
-      <c r="S20" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="T20" t="n">
-        <v>3.38</v>
-      </c>
-      <c r="U20" t="n">
         <v>82.90000000000001</v>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="R20" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -1919,36 +1737,32 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
       <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
+      <c r="K21" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="L21" t="n">
+        <v>626.7</v>
+      </c>
       <c r="M21" t="n">
-        <v>1</v>
-      </c>
-      <c r="N21" t="inlineStr"/>
+        <v>86.45999999999999</v>
+      </c>
+      <c r="N21" t="n">
+        <v>66</v>
+      </c>
       <c r="O21" t="n">
-        <v>0.36</v>
+        <v>6.57</v>
       </c>
       <c r="P21" t="n">
-        <v>626.7</v>
+        <v>0.4</v>
       </c>
       <c r="Q21" t="n">
-        <v>86.45999999999999</v>
-      </c>
-      <c r="R21" t="n">
-        <v>66</v>
-      </c>
-      <c r="S21" t="n">
-        <v>6.57</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="U21" t="n">
         <v>31.6</v>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="R21" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -1987,36 +1801,32 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>2</v>
+      </c>
       <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L22" t="n">
+        <v>1675</v>
+      </c>
       <c r="M22" t="n">
-        <v>2</v>
-      </c>
-      <c r="N22" t="inlineStr"/>
+        <v>27.19</v>
+      </c>
+      <c r="N22" t="n">
+        <v>61</v>
+      </c>
       <c r="O22" t="n">
-        <v>0.93</v>
+        <v>1.02</v>
       </c>
       <c r="P22" t="n">
-        <v>1675</v>
+        <v>1.32</v>
       </c>
       <c r="Q22" t="n">
-        <v>27.19</v>
-      </c>
-      <c r="R22" t="n">
-        <v>61</v>
-      </c>
-      <c r="S22" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="T22" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="U22" t="n">
         <v>11.1</v>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="R22" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -2055,36 +1865,32 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
       <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L23" t="n">
+        <v>1715.8</v>
+      </c>
       <c r="M23" t="n">
-        <v>2</v>
-      </c>
-      <c r="N23" t="inlineStr"/>
+        <v>30.21</v>
+      </c>
+      <c r="N23" t="n">
+        <v>90</v>
+      </c>
       <c r="O23" t="n">
-        <v>0.7</v>
+        <v>1.95</v>
       </c>
       <c r="P23" t="n">
-        <v>1715.8</v>
+        <v>2.86</v>
       </c>
       <c r="Q23" t="n">
-        <v>30.21</v>
-      </c>
-      <c r="R23" t="n">
-        <v>90</v>
-      </c>
-      <c r="S23" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="T23" t="n">
-        <v>2.86</v>
-      </c>
-      <c r="U23" t="n">
         <v>10.6</v>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="R23" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -2105,27 +1911,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TWSE排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>大盤比重%</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>建議</t>
         </is>
@@ -2376,37 +2182,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TWSE排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>大盤比重%</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>是否0050</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>評等</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>估值</t>
         </is>
@@ -5717,27 +5523,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>比重%</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>市值億</t>
         </is>
@@ -7854,111 +7660,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>OTC排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>OTC市值億</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>納入潛力分</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>評等</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>品質總分</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>估值</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>未來估值</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>PEG</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>ForwardPE</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>成長率g%</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>改善訊號數</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>分級</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>含金量</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>PER(自算)</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>PE位階%</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>PBR</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>殖利率%</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>最新月營收年增%</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>循環股</t>
         </is>
@@ -7997,33 +7783,29 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L2" t="n">
+        <v>21</v>
+      </c>
       <c r="M2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
+        <v>56</v>
+      </c>
+      <c r="N2" t="n">
+        <v>7</v>
+      </c>
       <c r="O2" t="n">
-        <v>0.92</v>
+        <v>2.24</v>
       </c>
       <c r="P2" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>56</v>
-      </c>
-      <c r="R2" t="n">
-        <v>7</v>
-      </c>
-      <c r="S2" t="n">
-        <v>2.24</v>
-      </c>
-      <c r="T2" t="n">
         <v>58.3</v>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8062,33 +7844,29 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>3</v>
+      </c>
       <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="L3" t="n">
+        <v>20.19</v>
+      </c>
       <c r="M3" t="n">
-        <v>3</v>
-      </c>
-      <c r="N3" t="inlineStr"/>
+        <v>72</v>
+      </c>
+      <c r="N3" t="n">
+        <v>3.02</v>
+      </c>
       <c r="O3" t="n">
-        <v>1.53</v>
+        <v>4.43</v>
       </c>
       <c r="P3" t="n">
-        <v>20.19</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>72</v>
-      </c>
-      <c r="R3" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="S3" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="T3" t="n">
         <v>10.3</v>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8127,33 +7905,29 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>4</v>
+      </c>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="L4" t="n">
+        <v>35.84</v>
+      </c>
       <c r="M4" t="n">
-        <v>4</v>
-      </c>
-      <c r="N4" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="N4" t="n">
+        <v>3.82</v>
+      </c>
       <c r="O4" t="n">
-        <v>1.85</v>
+        <v>1.05</v>
       </c>
       <c r="P4" t="n">
-        <v>35.84</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>40</v>
-      </c>
-      <c r="R4" t="n">
-        <v>3.82</v>
-      </c>
-      <c r="S4" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="T4" t="n">
         <v>37</v>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8192,33 +7966,29 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="L5" t="n">
+        <v>27.9</v>
+      </c>
       <c r="M5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N5" t="inlineStr"/>
+        <v>91</v>
+      </c>
+      <c r="N5" t="n">
+        <v>8.57</v>
+      </c>
       <c r="O5" t="n">
-        <v>1.21</v>
+        <v>2.79</v>
       </c>
       <c r="P5" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>91</v>
-      </c>
-      <c r="R5" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="S5" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="T5" t="n">
         <v>15.4</v>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8226,139 +7996,121 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4506</t>
+          <t>5351</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>崇友</t>
+          <t>鈺創</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>210.6</v>
+        <v>298.9</v>
       </c>
       <c r="E6" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>91</v>
+        <v>53</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>🟡未來合理</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>1.27</v>
-      </c>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
-        <v>15.1</v>
+        <v>1.85</v>
       </c>
       <c r="L6" t="n">
-        <v>13.5</v>
+        <v>94.79000000000001</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
-      </c>
-      <c r="N6" t="inlineStr"/>
+        <v>85</v>
+      </c>
+      <c r="N6" t="n">
+        <v>6.29</v>
+      </c>
       <c r="O6" t="n">
-        <v>1.28</v>
+        <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>17.12</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>55</v>
-      </c>
-      <c r="R6" t="n">
-        <v>3.39</v>
-      </c>
-      <c r="S6" t="n">
-        <v>4.45</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="U6" t="inlineStr"/>
+        <v>605.5</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>⚠️循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5351</t>
+          <t>4506</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>鈺創</t>
+          <t>崇友</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>298.9</v>
+        <v>210.6</v>
       </c>
       <c r="E7" t="n">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>53</v>
+        <v>91</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
+          <t>🟠偏貴</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>3</v>
+      </c>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="L7" t="n">
+        <v>17.12</v>
+      </c>
       <c r="M7" t="n">
-        <v>3</v>
-      </c>
-      <c r="N7" t="inlineStr"/>
+        <v>55</v>
+      </c>
+      <c r="N7" t="n">
+        <v>3.39</v>
+      </c>
       <c r="O7" t="n">
-        <v>1.85</v>
+        <v>4.45</v>
       </c>
       <c r="P7" t="n">
-        <v>94.79000000000001</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>85</v>
-      </c>
-      <c r="R7" t="n">
-        <v>6.29</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>605.5</v>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>⚠️循環(看PBR)</t>
-        </is>
-      </c>
+        <v>0.6</v>
+      </c>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8393,43 +8145,29 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>🔴未來過熱</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>1.03</v>
-      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
-        <v>38.8</v>
+        <v>1.15</v>
       </c>
       <c r="L8" t="n">
-        <v>60</v>
+        <v>62.01</v>
       </c>
       <c r="M8" t="n">
-        <v>3</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
+        <v>83</v>
+      </c>
+      <c r="N8" t="n">
+        <v>32.45</v>
+      </c>
       <c r="O8" t="n">
-        <v>1.15</v>
+        <v>1.09</v>
       </c>
       <c r="P8" t="n">
-        <v>62.01</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>83</v>
-      </c>
-      <c r="R8" t="n">
-        <v>32.45</v>
-      </c>
-      <c r="S8" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="T8" t="n">
         <v>99.3</v>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8464,33 +8202,29 @@
           <t>🟢便宜</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
+      <c r="K9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2.62</v>
+      </c>
       <c r="M9" t="n">
-        <v>3</v>
-      </c>
-      <c r="N9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.98</v>
+      </c>
       <c r="O9" t="n">
-        <v>0.01</v>
+        <v>6.03</v>
       </c>
       <c r="P9" t="n">
-        <v>2.62</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>1</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="S9" t="n">
-        <v>6.03</v>
-      </c>
-      <c r="T9" t="n">
         <v>8.1</v>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8529,43 +8263,29 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>🟠未來偏貴</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>3.69</v>
-      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
-        <v>26.3</v>
+        <v>1.13</v>
       </c>
       <c r="L10" t="n">
-        <v>7.7</v>
+        <v>28.33</v>
       </c>
       <c r="M10" t="n">
-        <v>3</v>
-      </c>
-      <c r="N10" t="inlineStr"/>
+        <v>74</v>
+      </c>
+      <c r="N10" t="n">
+        <v>17.29</v>
+      </c>
       <c r="O10" t="n">
-        <v>1.13</v>
+        <v>3.21</v>
       </c>
       <c r="P10" t="n">
-        <v>28.33</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>74</v>
-      </c>
-      <c r="R10" t="n">
-        <v>17.29</v>
-      </c>
-      <c r="S10" t="n">
-        <v>3.21</v>
-      </c>
-      <c r="T10" t="n">
         <v>23.8</v>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -8600,41 +8320,29 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>🔴未來過熱</t>
-        </is>
+      <c r="I11" t="n">
+        <v>2</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>36</v>
+        <v>1.67</v>
       </c>
       <c r="L11" t="n">
-        <v>-5.7</v>
+        <v>33.95</v>
       </c>
       <c r="M11" t="n">
-        <v>2</v>
-      </c>
-      <c r="N11" t="inlineStr"/>
+        <v>100</v>
+      </c>
+      <c r="N11" t="n">
+        <v>4.37</v>
+      </c>
       <c r="O11" t="n">
-        <v>1.67</v>
+        <v>2.12</v>
       </c>
       <c r="P11" t="n">
-        <v>33.95</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>100</v>
-      </c>
-      <c r="R11" t="n">
-        <v>4.37</v>
-      </c>
-      <c r="S11" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="T11" t="n">
         <v>22.1</v>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8669,33 +8377,29 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>2</v>
+      </c>
       <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="L12" t="n">
+        <v>58.01</v>
+      </c>
       <c r="M12" t="n">
-        <v>2</v>
-      </c>
-      <c r="N12" t="inlineStr"/>
+        <v>100</v>
+      </c>
+      <c r="N12" t="n">
+        <v>4.14</v>
+      </c>
       <c r="O12" t="n">
-        <v>2.14</v>
+        <v>1.51</v>
       </c>
       <c r="P12" t="n">
-        <v>58.01</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R12" t="n">
-        <v>4.14</v>
-      </c>
-      <c r="S12" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="T12" t="n">
         <v>11.8</v>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8734,33 +8438,29 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
       <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L13" t="n">
+        <v>25.88</v>
+      </c>
       <c r="M13" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" t="inlineStr"/>
+        <v>100</v>
+      </c>
+      <c r="N13" t="n">
+        <v>5.6</v>
+      </c>
       <c r="O13" t="n">
-        <v>0.92</v>
+        <v>2.72</v>
       </c>
       <c r="P13" t="n">
-        <v>25.88</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>100</v>
-      </c>
-      <c r="R13" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="S13" t="n">
-        <v>2.72</v>
-      </c>
-      <c r="T13" t="n">
         <v>81.7</v>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8799,33 +8499,29 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
       <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="L14" t="n">
+        <v>64.42</v>
+      </c>
       <c r="M14" t="n">
-        <v>1</v>
-      </c>
-      <c r="N14" t="inlineStr"/>
+        <v>71</v>
+      </c>
+      <c r="N14" t="n">
+        <v>9.17</v>
+      </c>
       <c r="O14" t="n">
-        <v>0.68</v>
+        <v>1.43</v>
       </c>
       <c r="P14" t="n">
-        <v>64.42</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>71</v>
-      </c>
-      <c r="R14" t="n">
-        <v>9.17</v>
-      </c>
-      <c r="S14" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="T14" t="n">
         <v>-43.4</v>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8833,23 +8529,23 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6803</t>
+          <t>5371</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>中光電</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>208.6</v>
+        <v>299.1</v>
       </c>
       <c r="E15" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -8857,70 +8553,60 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>🟡合理</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>🟢未來便宜</t>
-        </is>
-      </c>
-      <c r="J15" t="n">
-        <v>2.52</v>
-      </c>
+          <t>🟠偏貴</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
-        <v>14.7</v>
+        <v>3.75</v>
       </c>
       <c r="L15" t="n">
-        <v>6.2</v>
+        <v>127.5</v>
       </c>
       <c r="M15" t="n">
-        <v>2</v>
-      </c>
-      <c r="N15" t="inlineStr"/>
+        <v>100</v>
+      </c>
+      <c r="N15" t="n">
+        <v>1.13</v>
+      </c>
       <c r="O15" t="n">
-        <v>-0.87</v>
+        <v>0.65</v>
       </c>
       <c r="P15" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>2</v>
-      </c>
-      <c r="R15" t="n">
-        <v>3.33</v>
-      </c>
-      <c r="S15" t="n">
-        <v>5.48</v>
-      </c>
-      <c r="T15" t="n">
-        <v>-4.3</v>
-      </c>
-      <c r="U15" t="inlineStr"/>
+        <v>6.1</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>⚠️循環(看PBR)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>5371</t>
+          <t>8064</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>中光電</t>
+          <t>東捷</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>299.1</v>
+        <v>288.3</v>
       </c>
       <c r="E16" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -8928,40 +8614,36 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr"/>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>2</v>
+      </c>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="L16" t="n">
+        <v>70.13</v>
+      </c>
       <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="inlineStr"/>
+        <v>79</v>
+      </c>
+      <c r="N16" t="n">
+        <v>7.07</v>
+      </c>
       <c r="O16" t="n">
-        <v>3.75</v>
+        <v>0.59</v>
       </c>
       <c r="P16" t="n">
-        <v>127.5</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>100</v>
-      </c>
-      <c r="R16" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="S16" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="T16" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="U16" t="inlineStr">
+        <v>-17.5</v>
+      </c>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -8969,20 +8651,20 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>8064</t>
+          <t>3587</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>東捷</t>
+          <t>閎康</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>288.3</v>
+        <v>217.4</v>
       </c>
       <c r="E17" t="n">
         <v>38</v>
@@ -8993,40 +8675,36 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>2</v>
+      </c>
       <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="L17" t="n">
+        <v>40.16</v>
+      </c>
       <c r="M17" t="n">
-        <v>2</v>
-      </c>
-      <c r="N17" t="inlineStr"/>
+        <v>97</v>
+      </c>
+      <c r="N17" t="n">
+        <v>4.01</v>
+      </c>
       <c r="O17" t="n">
-        <v>1.14</v>
+        <v>1.48</v>
       </c>
       <c r="P17" t="n">
-        <v>70.13</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>79</v>
-      </c>
-      <c r="R17" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="S17" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="T17" t="n">
-        <v>-17.5</v>
-      </c>
-      <c r="U17" t="inlineStr">
+        <v>26.9</v>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -9034,23 +8712,23 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3587</t>
+          <t>6803</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>閎康</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>217.4</v>
+        <v>208.6</v>
       </c>
       <c r="E18" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -9058,44 +8736,36 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>🟡合理</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+      <c r="K18" t="n">
+        <v>-0.87</v>
+      </c>
+      <c r="L18" t="n">
+        <v>15.6</v>
+      </c>
       <c r="M18" t="n">
         <v>2</v>
       </c>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" t="n">
+        <v>3.33</v>
+      </c>
       <c r="O18" t="n">
-        <v>3.9</v>
+        <v>5.48</v>
       </c>
       <c r="P18" t="n">
-        <v>40.16</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>97</v>
-      </c>
-      <c r="R18" t="n">
-        <v>4.01</v>
-      </c>
-      <c r="S18" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="T18" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>⚠️循環(看PBR)</t>
-        </is>
-      </c>
+        <v>-4.3</v>
+      </c>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -9130,33 +8800,29 @@
           <t>🔴過熱</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
       <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>-3.66</v>
+      </c>
+      <c r="L19" t="n">
+        <v>251.19</v>
+      </c>
       <c r="M19" t="n">
-        <v>1</v>
-      </c>
-      <c r="N19" t="inlineStr"/>
+        <v>93</v>
+      </c>
+      <c r="N19" t="n">
+        <v>9.4</v>
+      </c>
       <c r="O19" t="n">
-        <v>-3.66</v>
+        <v>0</v>
       </c>
       <c r="P19" t="n">
-        <v>251.19</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>93</v>
-      </c>
-      <c r="R19" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="S19" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" t="n">
         <v>140.2</v>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -9195,33 +8861,29 @@
           <t>🟠偏貴</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
       <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>-0.67</v>
+      </c>
+      <c r="L20" t="n">
+        <v>65.81999999999999</v>
+      </c>
       <c r="M20" t="n">
+        <v>52</v>
+      </c>
+      <c r="N20" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="O20" t="n">
         <v>0</v>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="n">
-        <v>-0.67</v>
-      </c>
       <c r="P20" t="n">
-        <v>65.81999999999999</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>52</v>
-      </c>
-      <c r="R20" t="n">
-        <v>8.01</v>
-      </c>
-      <c r="S20" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" t="n">
         <v>-13.9</v>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -9242,27 +8904,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>OTC排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>市值億</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>建議</t>
         </is>
@@ -9766,27 +9428,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>收盤</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>市值億</t>
         </is>
@@ -11907,32 +11569,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>OTC排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>市值億</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>轉上市定位</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>在我們PICKS</t>
         </is>
@@ -12289,12 +11951,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>值</t>
         </is>

</xml_diff>

<commit_message>
data: 0050 納入預測 20260625
</commit_message>
<xml_diff>
--- a/data/台股_0050納入預測.xlsx
+++ b/data/台股_0050納入預測.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W23"/>
+  <dimension ref="A1:W24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1844,23 +1844,23 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6415</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>和碩</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.1605</v>
+        <v>0.1632</v>
       </c>
       <c r="E19" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1868,7 +1868,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1887,29 +1887,29 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
-        <v>0.36</v>
+        <v>2.28</v>
       </c>
       <c r="Q19" t="n">
-        <v>626.7</v>
+        <v>2306.6</v>
       </c>
       <c r="R19" t="n">
-        <v>86.45999999999999</v>
+        <v>19.77</v>
       </c>
       <c r="S19" t="n">
-        <v>66</v>
+        <v>99</v>
       </c>
       <c r="T19" t="n">
-        <v>6.57</v>
+        <v>1.14</v>
       </c>
       <c r="U19" t="n">
-        <v>0.4</v>
+        <v>4.66</v>
       </c>
       <c r="V19" t="n">
-        <v>31.6</v>
+        <v>12</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
@@ -1919,23 +1919,23 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3702</t>
+          <t>6415</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>大聯大</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.1357</v>
+        <v>0.1605</v>
       </c>
       <c r="E20" t="n">
-        <v>30.5</v>
+        <v>35</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1959,32 +1959,32 @@
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
-        <v>-0.89</v>
+        <v>0.36</v>
       </c>
       <c r="Q20" t="n">
-        <v>1889</v>
+        <v>626.7</v>
       </c>
       <c r="R20" t="n">
-        <v>14.17</v>
+        <v>86.45999999999999</v>
       </c>
       <c r="S20" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="T20" t="n">
-        <v>2.1</v>
+        <v>6.57</v>
       </c>
       <c r="U20" t="n">
-        <v>3.38</v>
+        <v>0.4</v>
       </c>
       <c r="V20" t="n">
-        <v>82.90000000000001</v>
+        <v>31.6</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
@@ -1994,23 +1994,23 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3034</t>
+          <t>3702</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>聯詠</t>
+          <t>大聯大</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.1996</v>
+        <v>0.1357</v>
       </c>
       <c r="E21" t="n">
-        <v>26</v>
+        <v>30.5</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -2018,7 +2018,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2034,32 +2034,32 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>-10</v>
+        <v>-5</v>
       </c>
       <c r="N21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
-        <v>1.01</v>
+        <v>-0.89</v>
       </c>
       <c r="Q21" t="n">
-        <v>3310.3</v>
+        <v>1889</v>
       </c>
       <c r="R21" t="n">
-        <v>22.29</v>
+        <v>14.17</v>
       </c>
       <c r="S21" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="T21" t="n">
-        <v>4.6</v>
+        <v>2.1</v>
       </c>
       <c r="U21" t="n">
-        <v>4.23</v>
+        <v>3.38</v>
       </c>
       <c r="V21" t="n">
-        <v>9.4</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
@@ -2069,20 +2069,20 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>1605</t>
+          <t>3034</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>華新</t>
+          <t>聯詠</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.1181</v>
+        <v>0.1996</v>
       </c>
       <c r="E22" t="n">
         <v>26</v>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2109,32 +2109,32 @@
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="N22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
-        <v>0.93</v>
+        <v>1.01</v>
       </c>
       <c r="Q22" t="n">
-        <v>1675</v>
+        <v>3310.3</v>
       </c>
       <c r="R22" t="n">
-        <v>27.19</v>
+        <v>22.29</v>
       </c>
       <c r="S22" t="n">
-        <v>61</v>
+        <v>97</v>
       </c>
       <c r="T22" t="n">
-        <v>1.02</v>
+        <v>4.6</v>
       </c>
       <c r="U22" t="n">
-        <v>1.32</v>
+        <v>4.23</v>
       </c>
       <c r="V22" t="n">
-        <v>11.1</v>
+        <v>9.4</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
@@ -2144,23 +2144,23 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1504</t>
+          <t>1605</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>東元</t>
+          <t>華新</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.1226</v>
+        <v>0.1181</v>
       </c>
       <c r="E23" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -2168,11 +2168,11 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2191,27 +2191,102 @@
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>1675</v>
+      </c>
+      <c r="R23" t="n">
+        <v>27.19</v>
+      </c>
+      <c r="S23" t="n">
+        <v>61</v>
+      </c>
+      <c r="T23" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="U23" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="V23" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>⚠️循環(看PBR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>88</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1504</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>東元</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0.1226</v>
+      </c>
+      <c r="E24" t="n">
+        <v>16</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>36</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>⏸ 循環(看PBR)</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>2</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="n">
         <v>0.7</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="Q24" t="n">
         <v>1715.8</v>
       </c>
-      <c r="R23" t="n">
+      <c r="R24" t="n">
         <v>30.21</v>
       </c>
-      <c r="S23" t="n">
+      <c r="S24" t="n">
         <v>90</v>
       </c>
-      <c r="T23" t="n">
+      <c r="T24" t="n">
         <v>1.95</v>
       </c>
-      <c r="U23" t="n">
+      <c r="U24" t="n">
         <v>2.86</v>
       </c>
-      <c r="V23" t="n">
+      <c r="V24" t="n">
         <v>10.6</v>
       </c>
-      <c r="W23" t="inlineStr">
+      <c r="W24" t="inlineStr">
         <is>
           <t>⚠️循環(看PBR)</t>
         </is>
@@ -2228,7 +2303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2283,20 +2358,20 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>2615</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>和碩</t>
+          <t>萬海</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.1632</v>
+        <v>0.1582</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2306,20 +2381,20 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2615</t>
+          <t>2618</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>萬海</t>
+          <t>長榮航</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.1582</v>
+        <v>0.1339</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2329,20 +2404,20 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2618</t>
+          <t>6531</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>長榮航</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.1339</v>
+        <v>0.1331</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2352,20 +2427,20 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6531</t>
+          <t>5876</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>上海商銀</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.1331</v>
+        <v>0.1329</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -2375,20 +2450,20 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5876</t>
+          <t>2492</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>上海商銀</t>
+          <t>華新科</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.1329</v>
+        <v>0.1316</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2398,20 +2473,20 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2492</t>
+          <t>2609</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>華新科</t>
+          <t>陽明</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.1316</v>
+        <v>0.1265</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -2421,20 +2496,20 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2609</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>陽明</t>
+          <t>台泥</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.1265</v>
+        <v>0.1262</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2444,45 +2519,22 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>2409</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>台泥</t>
+          <t>友達</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.1262</v>
+        <v>0.1194</v>
       </c>
       <c r="E10" t="inlineStr">
-        <is>
-          <t>加入 PICKS 抓體檢</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>89</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2409</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>友達</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>0.1194</v>
-      </c>
-      <c r="E11" t="inlineStr">
         <is>
           <t>加入 PICKS 抓體檢</t>
         </is>
@@ -2499,7 +2551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3099,20 +3151,20 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2887</t>
+          <t>2886</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>台新新光金</t>
+          <t>兆豐金</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.3992</v>
+        <v>0.408</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3121,7 +3173,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -3132,25 +3184,29 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2357</t>
+          <t>2887</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>華碩</t>
+          <t>台新新光金</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.3887</v>
-      </c>
-      <c r="E21" t="inlineStr"/>
+        <v>0.3992</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -3161,29 +3217,25 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>4958</t>
+          <t>2357</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>華碩</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.3791</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.3887</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3194,20 +3246,20 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>8046</t>
+          <t>4958</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>南電</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.3768</v>
+        <v>0.3791</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3216,7 +3268,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3227,20 +3279,20 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>8046</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>光寶科</t>
+          <t>南電</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.3736</v>
+        <v>0.3768</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3249,7 +3301,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -3260,25 +3312,29 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>3653</t>
+          <t>2301</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>健策</t>
+          <t>光寶科</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.3577</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
+        <v>0.3736</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3289,53 +3345,49 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>3653</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>玉山金</t>
+          <t>健策</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.3442</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.3577</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6505</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>台塑化</t>
+          <t>玉山金</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.3367</v>
+        <v>0.3442</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -3344,69 +3396,69 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>6505</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>台塑化</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.3319</v>
-      </c>
-      <c r="E28" t="inlineStr"/>
+        <v>0.3367</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>2059</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>大立光</t>
+          <t>川湖</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.3226</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.3319</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -3417,20 +3469,20 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>永豐金</t>
+          <t>大立光</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.2989</v>
+        <v>0.3226</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -3439,7 +3491,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3450,20 +3502,20 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>2890</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>研華</t>
+          <t>永豐金</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.2947</v>
+        <v>0.2989</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -3472,7 +3524,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3483,20 +3535,20 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2880</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>華南金</t>
+          <t>研華</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.2919</v>
+        <v>0.2947</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -3505,7 +3557,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3516,20 +3568,20 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>3045</t>
+          <t>2880</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>台灣大</t>
+          <t>華南金</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.2854</v>
+        <v>0.2919</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -3538,69 +3590,69 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>3481</t>
+          <t>3045</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>台灣大</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.2802</v>
-      </c>
-      <c r="E34" t="inlineStr"/>
+        <v>0.2854</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>3665</t>
+          <t>3481</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>貿聯-KY</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.2797</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2802</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3611,25 +3663,29 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>3189</t>
+          <t>3665</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>貿聯-KY</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.2641</v>
-      </c>
-      <c r="E36" t="inlineStr"/>
+        <v>0.2797</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3640,29 +3696,25 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2883</t>
+          <t>3189</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>凱基金</t>
+          <t>景碩</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.2626</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2641</v>
+      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3673,25 +3725,29 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>6770</t>
+          <t>2883</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>力積電</t>
+          <t>凱基金</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.2577</v>
-      </c>
-      <c r="E38" t="inlineStr"/>
+        <v>0.2626</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3702,25 +3758,25 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>3036</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>文曄</t>
+          <t>力積電</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.251</v>
+        <v>0.2577</v>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3731,141 +3787,145 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>6446</t>
+          <t>3036</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>藥華藥</t>
+          <t>文曄</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.2429</v>
+        <v>0.251</v>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>3661</t>
+          <t>5880</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>世芯-KY</t>
+          <t>合庫金</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.2408</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
+        <v>0.2464</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2313</t>
+          <t>6446</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>華通</t>
+          <t>藥華藥</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.2331</v>
+        <v>0.2429</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>4904</t>
+          <t>3661</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>遠傳</t>
+          <t>世芯-KY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.2285</v>
+        <v>0.2408</v>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2337</t>
+          <t>2313</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>旺宏</t>
+          <t>華通</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.2211</v>
+        <v>0.2331</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3876,25 +3936,25 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>6515</t>
+          <t>4904</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>遠傳</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.2147</v>
+        <v>0.2285</v>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3905,29 +3965,25 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2379</t>
+          <t>2337</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>瑞昱</t>
+          <t>旺宏</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.2056</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2211</v>
+      </c>
+      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3938,20 +3994,20 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>3533</t>
+          <t>6515</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>嘉澤</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.2051</v>
+        <v>0.2147</v>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
@@ -3967,54 +4023,58 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>3034</t>
+          <t>2379</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>聯詠</t>
+          <t>瑞昱</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.1996</v>
-      </c>
-      <c r="E48" t="inlineStr"/>
+        <v>0.2056</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>6239</t>
+          <t>3533</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>嘉澤</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.1978</v>
+        <v>0.2051</v>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4025,25 +4085,25 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>3034</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>亞德客-KY</t>
+          <t>聯詠</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.1925</v>
+        <v>0.1996</v>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4054,25 +4114,25 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1519</t>
+          <t>6239</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>華城</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.1898</v>
+        <v>0.1978</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4083,87 +4143,83 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>3044</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>健鼎</t>
+          <t>亞德客-KY</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.1883</v>
+        <v>0.1925</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2207</t>
+          <t>1519</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>和泰車</t>
+          <t>華城</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.185</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.1898</v>
+      </c>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2356</t>
+          <t>3044</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>英業達</t>
+          <t>健鼎</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.1732</v>
+        <v>0.1883</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4174,25 +4230,29 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2376</t>
+          <t>2207</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>技嘉</t>
+          <t>和泰車</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.1704</v>
-      </c>
-      <c r="E55" t="inlineStr"/>
+        <v>0.185</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4203,58 +4263,54 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>6415</t>
+          <t>2356</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>英業達</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.1605</v>
+        <v>0.1732</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2912</t>
+          <t>2376</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>統一超</t>
+          <t>技嘉</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.153</v>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.1704</v>
+      </c>
+      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4265,107 +4321,111 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2404</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>漢唐</t>
+          <t>和碩</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.1514</v>
+        <v>0.1632</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>1802</t>
+          <t>6415</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>台玻</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.1438</v>
+        <v>0.1605</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>3702</t>
+          <t>2912</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>大聯大</t>
+          <t>統一超</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.1357</v>
-      </c>
-      <c r="E60" t="inlineStr"/>
+        <v>0.153</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>6139</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>亞翔</t>
+          <t>漢唐</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.127</v>
+        <v>0.1514</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
@@ -4381,25 +4441,25 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>1504</t>
+          <t>1802</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>東元</t>
+          <t>台玻</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.1226</v>
+        <v>0.1438</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -4410,20 +4470,20 @@
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>1605</t>
+          <t>3702</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>華新</t>
+          <t>大聯大</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.1181</v>
+        <v>0.1357</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
@@ -4439,20 +4499,20 @@
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>6139</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>勤誠</t>
+          <t>亞翔</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.1176</v>
+        <v>0.127</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
@@ -4468,83 +4528,83 @@
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2451</t>
+          <t>1504</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>創見</t>
+          <t>東元</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.1001</v>
+        <v>0.1226</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>6442</t>
+          <t>1605</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>華新</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.099</v>
+        <v>0.1181</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>8210</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>上銀</t>
+          <t>勤誠</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.0946</v>
+        <v>0.1176</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -4555,20 +4615,20 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>1503</t>
+          <t>2451</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>士電</t>
+          <t>創見</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.0784</v>
+        <v>0.1001</v>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
@@ -4578,60 +4638,60 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2812</t>
+          <t>6442</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>台中銀</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.0764</v>
+        <v>0.099</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>6257</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>矽格</t>
+          <t>上銀</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.0757</v>
+        <v>0.0946</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -4642,83 +4702,83 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>5269</t>
+          <t>3532</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>祥碩</t>
+          <t>台勝科</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.07530000000000001</v>
+        <v>0.0851</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2353</t>
+          <t>1503</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>宏碁</t>
+          <t>士電</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.0738</v>
+        <v>0.0784</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>3026</t>
+          <t>6196</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>禾伸堂</t>
+          <t>帆宣</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.0731</v>
+        <v>0.0774</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -4729,54 +4789,54 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>1560</t>
+          <t>2812</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>中砂</t>
+          <t>台中銀</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.0727</v>
+        <v>0.0764</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8996</t>
+          <t>6257</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>高力</t>
+          <t>矽格</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.0693</v>
+        <v>0.0757</v>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -4787,83 +4847,83 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2467</t>
+          <t>5269</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>志聖</t>
+          <t>祥碩</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.0667</v>
+        <v>0.07530000000000001</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>3030</t>
+          <t>2353</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>德律</t>
+          <t>宏碁</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.0658</v>
+        <v>0.0738</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>5434</t>
+          <t>3026</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>崇越</t>
+          <t>禾伸堂</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.0599</v>
+        <v>0.0731</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4874,20 +4934,20 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>1513</t>
+          <t>1560</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>中興電</t>
+          <t>中砂</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.0576</v>
+        <v>0.0727</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
@@ -4897,31 +4957,31 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>6005</t>
+          <t>8996</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>群益證</t>
+          <t>高力</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.0575</v>
+        <v>0.0693</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4932,25 +4992,25 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>8150</t>
+          <t>2467</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>南茂</t>
+          <t>志聖</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.0547</v>
+        <v>0.0667</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4961,25 +5021,25 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2455</t>
+          <t>3030</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>全新</t>
+          <t>德律</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.0537</v>
+        <v>0.0658</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4990,25 +5050,25 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2855</t>
+          <t>5434</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>統一證</t>
+          <t>崇越</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.0523</v>
+        <v>0.0599</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -5019,25 +5079,25 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>3023</t>
+          <t>1513</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>信邦</t>
+          <t>中興電</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.0521</v>
+        <v>0.0576</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -5048,25 +5108,25 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>3450</t>
+          <t>6005</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>聯鈞</t>
+          <t>群益證</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0.0491</v>
+        <v>0.0575</v>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -5077,54 +5137,54 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>3583</t>
+          <t>8150</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>辛耘</t>
+          <t>南茂</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.0479</v>
+        <v>0.0547</v>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>3406</t>
+          <t>2455</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>玉晶光</t>
+          <t>全新</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.0467</v>
+        <v>0.0537</v>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -5135,49 +5195,49 @@
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>158</v>
+        <v>141</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>3005</t>
+          <t>2855</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>神基</t>
+          <t>統一證</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.0445</v>
+        <v>0.0523</v>
       </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2371</t>
+          <t>3023</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>大同</t>
+          <t>信邦</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.0441</v>
+        <v>0.0521</v>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
@@ -5187,26 +5247,26 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2645</t>
+          <t>6944</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>長榮航太</t>
+          <t>兆聯實業</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.0429</v>
+        <v>0.0499</v>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
@@ -5222,25 +5282,25 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>6451</t>
+          <t>3450</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>訊芯-KY</t>
+          <t>聯鈞</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.0426</v>
+        <v>0.0491</v>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -5251,25 +5311,25 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>172</v>
+        <v>150</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>4583</t>
+          <t>3583</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>台灣精銳</t>
+          <t>辛耘</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.0396</v>
+        <v>0.0479</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -5280,20 +5340,20 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>177</v>
+        <v>153</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>1773</t>
+          <t>3406</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>勝一</t>
+          <t>玉晶光</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.0385</v>
+        <v>0.0467</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
@@ -5309,78 +5369,78 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>8926</t>
+          <t>3005</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>台汽電</t>
+          <t>神基</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.038</v>
+        <v>0.0445</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2889</t>
+          <t>2371</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>國票金</t>
+          <t>大同</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.0367</v>
+        <v>0.0441</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>189</v>
+        <v>161</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>9917</t>
+          <t>2645</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>中保科</t>
+          <t>長榮航太</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.0354</v>
+        <v>0.0429</v>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
@@ -5390,26 +5450,26 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>196</v>
+        <v>164</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>3715</t>
+          <t>6451</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>定穎投控</t>
+          <t>訊芯-KY</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.0338</v>
+        <v>0.0426</v>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
@@ -5425,20 +5485,20 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>200</v>
+        <v>172</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2915</t>
+          <t>4583</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>潤泰全</t>
+          <t>台灣精銳</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.0334</v>
+        <v>0.0396</v>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
@@ -5448,31 +5508,31 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>531</v>
+        <v>177</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>3535</t>
+          <t>1773</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>晶彩科</t>
+          <t>勝一</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.0067</v>
+        <v>0.0385</v>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -5483,107 +5543,107 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>532</v>
+        <v>178</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>8341</t>
+          <t>8926</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>日友</t>
+          <t>台汽電</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.0067</v>
+        <v>0.038</v>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>560</v>
+        <v>180</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>3504</t>
+          <t>2889</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>揚明光</t>
+          <t>國票金</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.0061</v>
+        <v>0.0367</v>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>584</v>
+        <v>189</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>6863</t>
+          <t>9917</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>永道-KY</t>
+          <t>中保科</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.0056</v>
+        <v>0.0354</v>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>587</v>
+        <v>196</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>3004</t>
+          <t>3715</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>豐達科</t>
+          <t>定穎投控</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.0055</v>
+        <v>0.0338</v>
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
@@ -5593,26 +5653,26 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>589</v>
+        <v>200</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>7730</t>
+          <t>2915</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>暉盛-創</t>
+          <t>潤泰全</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.0054</v>
+        <v>0.0334</v>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
@@ -5622,26 +5682,26 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>590</v>
+        <v>531</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>9918</t>
+          <t>3535</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>欣天然</t>
+          <t>晶彩科</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.0054</v>
+        <v>0.0067</v>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
@@ -5651,26 +5711,26 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>613</v>
+        <v>532</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>3130</t>
+          <t>8341</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>一零四</t>
+          <t>日友</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.005</v>
+        <v>0.0067</v>
       </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
@@ -5686,107 +5746,107 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>655</v>
+        <v>541</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>4746</t>
+          <t>5292</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>台耀</t>
+          <t>華懋</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.0043</v>
+        <v>0.0065</v>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>661</v>
+        <v>560</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2453</t>
+          <t>3504</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>凌群</t>
+          <t>揚明光</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.0042</v>
+        <v>0.0061</v>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>695</v>
+        <v>572</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>6776</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>中鋼構</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.0037</v>
+        <v>0.0058</v>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>701</v>
+        <v>584</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>6112</t>
+          <t>6863</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>邁達特</t>
+          <t>永道-KY</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0.0036</v>
+        <v>0.0056</v>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
@@ -5796,26 +5856,26 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>710</v>
+        <v>587</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>5203</t>
+          <t>3004</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>訊連</t>
+          <t>豐達科</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.0035</v>
+        <v>0.0055</v>
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
@@ -5824,6 +5884,238 @@
         </is>
       </c>
       <c r="G111" t="inlineStr">
+        <is>
+          <t>🟠偏貴</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>589</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>7730</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>暉盛-創</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>590</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>9918</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>欣天然</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>🟠偏貴</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>613</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>3130</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>一零四</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>🟢便宜</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>655</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>4746</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>台耀</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>🟢便宜</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>661</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>2453</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>凌群</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>0.0042</v>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>🟢便宜</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>695</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>6776</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>展碁國際</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>🟠偏貴</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>701</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>6112</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>邁達特</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>🟠偏貴</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>710</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>5203</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>訊連</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>0.0035</v>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
         <is>
           <t>🟢便宜</t>
         </is>
@@ -12578,7 +12870,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6">
@@ -12588,7 +12880,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -12598,7 +12890,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -12608,7 +12900,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: 0050 納入預測 20260626
</commit_message>
<xml_diff>
--- a/data/台股_0050納入預測.xlsx
+++ b/data/台股_0050納入預測.xlsx
@@ -25,13 +25,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -50,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,117 +437,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TWSE排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>大盤比重%</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>納入潛力分</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>評等</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>品質總分</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>估值</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>未來估值</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PEG</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ForwardPE</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>成長率g%</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>⑪動態惡化扣分</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>改善訊號數</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>分級</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>含金量</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>市值(億)</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>PER(自算)</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>PE位階%</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>PBR</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>殖利率%</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>最新月營收年增%</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>循環股</t>
         </is>
@@ -1306,27 +1318,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TWSE排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>大盤比重%</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>建議</t>
         </is>
@@ -1343,41 +1355,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TWSE排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>大盤比重%</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>是否0050</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>評等</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>估值</t>
         </is>
@@ -1451,20 +1463,20 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3711</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>鴻海</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.8741</v>
+        <v>2.7827</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1484,20 +1496,20 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>3711</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.2615</v>
+        <v>1.8741</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1506,31 +1518,31 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3037</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>欣興</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.1429</v>
+        <v>1.2615</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1539,31 +1551,31 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2881</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>富邦金</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.0594</v>
+        <v>1.2498</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1572,7 +1584,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1583,20 +1595,20 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2327</t>
+          <t>3037</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>國巨*</t>
+          <t>欣興</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.0519</v>
+        <v>1.1429</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1605,7 +1617,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1616,20 +1628,20 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2345</t>
+          <t>2881</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>智邦</t>
+          <t>富邦金</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.9375</v>
+        <v>1.0594</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1638,7 +1650,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1649,20 +1661,20 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2882</t>
+          <t>2327</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>國泰金</t>
+          <t>國巨*</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.8643999999999999</v>
+        <v>1.0519</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1671,7 +1683,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1682,20 +1694,20 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2891</t>
+          <t>2345</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>中信金</t>
+          <t>智邦</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.8186</v>
+        <v>0.9375</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1704,7 +1716,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1715,20 +1727,20 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2408</t>
+          <t>2382</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>南亞科</t>
+          <t>廣達</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.7393</v>
+        <v>0.9004</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1737,7 +1749,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1748,20 +1760,20 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2360</t>
+          <t>2882</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>致茂</t>
+          <t>國泰金</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.7368</v>
+        <v>0.8643999999999999</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1770,7 +1782,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1781,20 +1793,20 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2412</t>
+          <t>2891</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>中華電</t>
+          <t>中信金</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.7308</v>
+        <v>0.8186</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1803,7 +1815,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1814,20 +1826,20 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3017</t>
+          <t>2408</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>奇鋐</t>
+          <t>南亞科</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.7186</v>
+        <v>0.7393</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1836,31 +1848,31 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2885</t>
+          <t>2360</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>元大金</t>
+          <t>致茂</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.5463</v>
+        <v>0.7368</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1869,7 +1881,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1880,20 +1892,20 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1303</t>
+          <t>2412</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>南亞</t>
+          <t>中華電</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.535</v>
+        <v>0.7308</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1902,7 +1914,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1913,20 +1925,20 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2344</t>
+          <t>3017</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>華邦電</t>
+          <t>奇鋐</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.4889</v>
+        <v>0.7186</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1935,31 +1947,31 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2368</t>
+          <t>2885</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>金像電</t>
+          <t>元大金</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.4634</v>
+        <v>0.5463</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1968,7 +1980,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1979,20 +1991,20 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3443</t>
+          <t>1303</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>創意</t>
+          <t>南亞</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.4303</v>
+        <v>0.535</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2001,7 +2013,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2012,20 +2024,20 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2886</t>
+          <t>2344</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>兆豐金</t>
+          <t>華邦電</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.408</v>
+        <v>0.4889</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2034,7 +2046,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2045,20 +2057,20 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2887</t>
+          <t>2368</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>台新新光金</t>
+          <t>金像電</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.3992</v>
+        <v>0.4634</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2067,7 +2079,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2078,20 +2090,20 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2357</t>
+          <t>3443</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>華碩</t>
+          <t>創意</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.3887</v>
+        <v>0.4303</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2100,7 +2112,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2111,20 +2123,20 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4958</t>
+          <t>2886</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>兆豐金</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.3791</v>
+        <v>0.408</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2133,7 +2145,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2144,20 +2156,20 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>8046</t>
+          <t>2887</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>南電</t>
+          <t>台新新光金</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.3768</v>
+        <v>0.3992</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2166,7 +2178,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2177,20 +2189,20 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>2357</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>光寶科</t>
+          <t>華碩</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.3736</v>
+        <v>0.3887</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2199,7 +2211,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2210,20 +2222,20 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>3653</t>
+          <t>4958</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>健策</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.3577</v>
+        <v>0.3791</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2232,7 +2244,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2243,20 +2255,20 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>8046</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>玉山金</t>
+          <t>南電</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.3442</v>
+        <v>0.3768</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2265,31 +2277,31 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6505</t>
+          <t>2301</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>台塑化</t>
+          <t>光寶科</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.3367</v>
+        <v>0.3736</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2303,26 +2315,26 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>3653</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>健策</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.3319</v>
+        <v>0.3577</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2342,20 +2354,20 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>大立光</t>
+          <t>玉山金</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.3226</v>
+        <v>0.3442</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2364,31 +2376,31 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>6505</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>永豐金</t>
+          <t>台塑化</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.2989</v>
+        <v>0.3367</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2397,31 +2409,31 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>2059</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>研華</t>
+          <t>川湖</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.2947</v>
+        <v>0.3319</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2430,7 +2442,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2441,20 +2453,20 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2880</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>華南金</t>
+          <t>大立光</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.2919</v>
+        <v>0.3226</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2463,7 +2475,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2474,20 +2486,20 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>3045</t>
+          <t>2890</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>台灣大</t>
+          <t>永豐金</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.2854</v>
+        <v>0.2989</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2496,31 +2508,31 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>1216</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>統一</t>
+          <t>研華</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.2805</v>
+        <v>0.2947</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2529,36 +2541,40 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>3481</t>
+          <t>2880</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>華南金</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.2802</v>
-      </c>
-      <c r="E37" t="inlineStr"/>
+        <v>0.2919</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2569,20 +2585,20 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>3665</t>
+          <t>3045</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>貿聯-KY</t>
+          <t>台灣大</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.2797</v>
+        <v>0.2854</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2596,64 +2612,64 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>3189</t>
+          <t>1216</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>統一</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.2641</v>
-      </c>
-      <c r="E39" t="inlineStr"/>
+        <v>0.2805</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2883</t>
+          <t>3481</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>凱基金</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.2626</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2802</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2664,25 +2680,29 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>6770</t>
+          <t>3665</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>力積電</t>
+          <t>貿聯-KY</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.2577</v>
-      </c>
-      <c r="E41" t="inlineStr"/>
+        <v>0.2797</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2693,20 +2713,20 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>3036</t>
+          <t>3189</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>文曄</t>
+          <t>景碩</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.251</v>
+        <v>0.2641</v>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
@@ -2722,20 +2742,20 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>5880</t>
+          <t>2883</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>合庫金</t>
+          <t>凱基金</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.2464</v>
+        <v>0.2626</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2749,61 +2769,57 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>6446</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>藥華藥</t>
+          <t>力積電</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.2429</v>
+        <v>0.2577</v>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>3661</t>
+          <t>3036</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>世芯-KY</t>
+          <t>文曄</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.2408</v>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.251</v>
+      </c>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>C</t>
@@ -2811,61 +2827,61 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2313</t>
+          <t>5880</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>華通</t>
+          <t>合庫金</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.2331</v>
-      </c>
-      <c r="E46" t="inlineStr"/>
+        <v>0.2464</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>4904</t>
+          <t>6446</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>遠傳</t>
+          <t>藥華藥</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.2285</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2429</v>
+      </c>
+      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>B</t>
@@ -2873,55 +2889,59 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2337</t>
+          <t>3661</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>旺宏</t>
+          <t>世芯-KY</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.2211</v>
-      </c>
-      <c r="E48" t="inlineStr"/>
+        <v>0.2408</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>6515</t>
+          <t>2313</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>華通</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.2147</v>
+        <v>0.2331</v>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
@@ -2937,49 +2957,53 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1301</t>
+          <t>4904</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>台塑</t>
+          <t>遠傳</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.2077</v>
-      </c>
-      <c r="E50" t="inlineStr"/>
+        <v>0.2285</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>2337</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>中鋼</t>
+          <t>旺宏</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.2066</v>
+        <v>0.2211</v>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
@@ -2989,31 +3013,31 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2379</t>
+          <t>6515</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>瑞昱</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.2056</v>
+        <v>0.2147</v>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3024,49 +3048,49 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>3533</t>
+          <t>1301</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>嘉澤</t>
+          <t>台塑</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.2051</v>
+        <v>0.2077</v>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1326</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>台化</t>
+          <t>中鋼</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.2011</v>
+        <v>0.2066</v>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
@@ -3076,60 +3100,60 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>3034</t>
+          <t>2379</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>聯詠</t>
+          <t>瑞昱</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.1996</v>
+        <v>0.2056</v>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>6239</t>
+          <t>3533</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>嘉澤</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.1978</v>
+        <v>0.2051</v>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3140,83 +3164,83 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>1326</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>亞德客-KY</t>
+          <t>台化</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.1925</v>
+        <v>0.2011</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1519</t>
+          <t>3034</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>華城</t>
+          <t>聯詠</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.1898</v>
+        <v>0.1996</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>3044</t>
+          <t>6239</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>健鼎</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.1883</v>
+        <v>0.1978</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3227,20 +3251,20 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2207</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>和泰車</t>
+          <t>亞德客-KY</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.185</v>
+        <v>0.1925</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
@@ -3250,31 +3274,31 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2356</t>
+          <t>1519</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>英業達</t>
+          <t>華城</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.1732</v>
+        <v>0.1898</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3285,112 +3309,112 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2376</t>
+          <t>3044</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>技嘉</t>
+          <t>健鼎</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.1704</v>
+        <v>0.1883</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>2207</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>和碩</t>
+          <t>和泰車</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.1632</v>
+        <v>0.185</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>6415</t>
+          <t>2356</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>英業達</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.1605</v>
+        <v>0.1732</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2912</t>
+          <t>2376</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>統一超</t>
+          <t>技嘉</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.153</v>
+        <v>0.1704</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3401,107 +3425,107 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2404</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>漢唐</t>
+          <t>和碩</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.1514</v>
+        <v>0.1632</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>1802</t>
+          <t>6415</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>台玻</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.1438</v>
+        <v>0.1605</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>3702</t>
+          <t>2912</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>大聯大</t>
+          <t>統一超</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.1357</v>
+        <v>0.153</v>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>6139</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>亞翔</t>
+          <t>漢唐</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.127</v>
+        <v>0.1514</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
@@ -3517,49 +3541,49 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>1802</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>台泥</t>
+          <t>台玻</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.1262</v>
+        <v>0.1438</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>1504</t>
+          <t>3702</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>東元</t>
+          <t>大聯大</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.1226</v>
+        <v>0.1357</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
@@ -3569,118 +3593,118 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>1605</t>
+          <t>6139</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>華新</t>
+          <t>亞翔</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.1181</v>
+        <v>0.127</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>勤誠</t>
+          <t>台泥</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.1176</v>
+        <v>0.1262</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2451</t>
+          <t>1504</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>創見</t>
+          <t>東元</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.1001</v>
+        <v>0.1226</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>6442</t>
+          <t>2409</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>友達</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.099</v>
+        <v>0.1194</v>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3691,20 +3715,20 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>1605</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>上銀</t>
+          <t>華新</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.0946</v>
+        <v>0.1181</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
@@ -3714,55 +3738,55 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>1402</t>
+          <t>8210</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>遠東新</t>
+          <t>勤誠</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.0944</v>
+        <v>0.1176</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3532</t>
+          <t>2324</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>台勝科</t>
+          <t>仁寶</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.0851</v>
+        <v>0.1112</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
@@ -3778,54 +3802,54 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>1102</t>
+          <t>2451</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>亞泥</t>
+          <t>創見</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.0829</v>
+        <v>0.1001</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>1503</t>
+          <t>6442</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>士電</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.0784</v>
+        <v>0.099</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3836,25 +3860,25 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>6196</t>
+          <t>2347</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>帆宣</t>
+          <t>聯強</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.0774</v>
+        <v>0.0985</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3865,28 +3889,202 @@
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2812</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>台中銀</t>
+          <t>上銀</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.0764</v>
+        <v>0.0946</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>102</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1402</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>遠東新</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>0.0944</v>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>🟢便宜</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>104</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>3532</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>台勝科</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>0.0851</v>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>105</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1102</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>亞泥</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>0.0829</v>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>🟢便宜</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>109</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>1503</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>士電</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>0.0784</v>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>110</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>6196</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>帆宣</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>0.0774</v>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>111</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2812</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>台中銀</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>0.0764</v>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr">
+        <is>
           <t>金融🏦</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
+      <c r="G88" t="inlineStr">
         <is>
           <t>🟠偏貴</t>
         </is>
@@ -3907,27 +4105,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>比重%</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>市值億</t>
         </is>
@@ -6048,112 +6246,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>OTC排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>OTC市值億</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>納入潛力分</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>評等</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>品質總分</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>估值</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>未來估值</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PEG</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ForwardPE</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>成長率g%</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>⑪動態惡化扣分</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>改善訊號數</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>分級</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>含金量</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>PER(自算)</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>PE位階%</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>PBR</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>殖利率%</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>最新月營收年增%</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>循環股</t>
         </is>
@@ -6978,27 +7176,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>OTC排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>市值億</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>建議</t>
         </is>
@@ -7226,27 +7424,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>收盤</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>市值億</t>
         </is>
@@ -9367,32 +9565,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>OTC排名</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>代號</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>名稱</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>市值億</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>轉上市定位</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>在我們PICKS</t>
         </is>
@@ -9581,12 +9779,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>值</t>
         </is>
@@ -9629,7 +9827,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
data: 0050 納入預測 20260629
</commit_message>
<xml_diff>
--- a/data/台股_0050納入預測.xlsx
+++ b/data/台股_0050納入預測.xlsx
@@ -1355,7 +1355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G106"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1991,20 +1991,20 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2885</t>
+          <t>6669</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>元大金</t>
+          <t>緯穎</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.5463</v>
+        <v>0.6958</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2013,31 +2013,31 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1303</t>
+          <t>2885</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>南亞</t>
+          <t>元大金</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.535</v>
+        <v>0.5463</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2057,20 +2057,20 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2344</t>
+          <t>1303</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>華邦電</t>
+          <t>南亞</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.4889</v>
+        <v>0.535</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2090,20 +2090,20 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2368</t>
+          <t>2344</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>金像電</t>
+          <t>華邦電</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.4634</v>
+        <v>0.4889</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2112,7 +2112,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2123,20 +2123,20 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>3443</t>
+          <t>2368</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>創意</t>
+          <t>金像電</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.4303</v>
+        <v>0.4634</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2156,20 +2156,20 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2886</t>
+          <t>3443</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>兆豐金</t>
+          <t>創意</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.408</v>
+        <v>0.4303</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2189,20 +2189,20 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2887</t>
+          <t>2886</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>台新新光金</t>
+          <t>兆豐金</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.3992</v>
+        <v>0.408</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2222,20 +2222,20 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2357</t>
+          <t>2887</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>華碩</t>
+          <t>台新新光金</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.3887</v>
+        <v>0.3992</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2255,20 +2255,20 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>4958</t>
+          <t>2357</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>華碩</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.3791</v>
+        <v>0.3887</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2288,20 +2288,20 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>8046</t>
+          <t>4958</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>南電</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.3768</v>
+        <v>0.3791</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2321,20 +2321,20 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>8046</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>光寶科</t>
+          <t>南電</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.3736</v>
+        <v>0.3768</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2354,20 +2354,20 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>3653</t>
+          <t>2301</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>健策</t>
+          <t>光寶科</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.3577</v>
+        <v>0.3736</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2387,20 +2387,20 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>3231</t>
+          <t>3653</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>緯創</t>
+          <t>健策</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.3466</v>
+        <v>0.3577</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2409,31 +2409,31 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2884</t>
+          <t>3231</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>玉山金</t>
+          <t>緯創</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.3442</v>
+        <v>0.3466</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2442,31 +2442,31 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6505</t>
+          <t>2884</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>台塑化</t>
+          <t>玉山金</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.3367</v>
+        <v>0.3442</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2475,31 +2475,31 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2059</t>
+          <t>6505</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>川湖</t>
+          <t>台塑化</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.3319</v>
+        <v>0.3367</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2508,31 +2508,31 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>2059</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>大立光</t>
+          <t>川湖</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.3226</v>
+        <v>0.3319</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2552,20 +2552,20 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2603</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>長榮</t>
+          <t>大立光</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.3171</v>
+        <v>0.3226</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2574,31 +2574,31 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2890</t>
+          <t>2603</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>永豐金</t>
+          <t>長榮</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.2989</v>
+        <v>0.3171</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2607,31 +2607,31 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>2890</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>研華</t>
+          <t>永豐金</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.2947</v>
+        <v>0.2989</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2651,20 +2651,20 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2880</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>華南金</t>
+          <t>研華</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.2919</v>
+        <v>0.2947</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2684,20 +2684,20 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>3045</t>
+          <t>2880</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>台灣大</t>
+          <t>華南金</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.2854</v>
+        <v>0.2919</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2706,31 +2706,31 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>1216</t>
+          <t>3045</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>統一</t>
+          <t>台灣大</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.2805</v>
+        <v>0.2854</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2750,22 +2750,26 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>3481</t>
+          <t>1216</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>統一</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.2802</v>
-      </c>
-      <c r="E43" t="inlineStr"/>
+        <v>0.2805</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>D</t>
@@ -2773,35 +2777,31 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>3665</t>
+          <t>3481</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>貿聯-KY</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.2797</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2802</v>
+      </c>
+      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2812,20 +2812,20 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2449</t>
+          <t>3665</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>京元電子</t>
+          <t>貿聯-KY</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.2762</v>
+        <v>0.2797</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2845,20 +2845,20 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2892</t>
+          <t>2449</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>第一金</t>
+          <t>京元電子</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.2714</v>
+        <v>0.2762</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2878,25 +2878,29 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>3189</t>
+          <t>2892</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>景碩</t>
+          <t>第一金</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.2641</v>
-      </c>
-      <c r="E47" t="inlineStr"/>
+        <v>0.2714</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2907,29 +2911,25 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2883</t>
+          <t>3189</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>凱基金</t>
+          <t>景碩</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.2626</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2641</v>
+      </c>
+      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2940,25 +2940,29 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>6770</t>
+          <t>2883</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>力積電</t>
+          <t>凱基金</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.2577</v>
-      </c>
-      <c r="E49" t="inlineStr"/>
+        <v>0.2626</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2969,25 +2973,25 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>3036</t>
+          <t>6770</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>文曄</t>
+          <t>力積電</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.251</v>
+        <v>0.2577</v>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2998,91 +3002,87 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>5880</t>
+          <t>3036</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>合庫金</t>
+          <t>文曄</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.2464</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.251</v>
+      </c>
+      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>6446</t>
+          <t>5880</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>藥華藥</t>
+          <t>合庫金</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.2429</v>
-      </c>
-      <c r="E52" t="inlineStr"/>
+        <v>0.2464</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>3661</t>
+          <t>6446</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>世芯-KY</t>
+          <t>藥華藥</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.2408</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2429</v>
+      </c>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3093,58 +3093,58 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2313</t>
+          <t>3661</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>華通</t>
+          <t>世芯-KY</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.2331</v>
-      </c>
-      <c r="E54" t="inlineStr"/>
+        <v>0.2408</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>4904</t>
+          <t>2313</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>遠傳</t>
+          <t>華通</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.2285</v>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0.2331</v>
+      </c>
+      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3155,25 +3155,29 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2337</t>
+          <t>4904</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>旺宏</t>
+          <t>遠傳</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.2211</v>
-      </c>
-      <c r="E56" t="inlineStr"/>
+        <v>0.2285</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3184,25 +3188,25 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>6515</t>
+          <t>2337</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>旺宏</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.2147</v>
+        <v>0.2211</v>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3213,49 +3217,49 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>1301</t>
+          <t>6515</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>台塑</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.2077</v>
+        <v>0.2147</v>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2002</t>
+          <t>1301</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>中鋼</t>
+          <t>台塑</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.2066</v>
+        <v>0.2077</v>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
@@ -3271,54 +3275,54 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2379</t>
+          <t>2002</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>瑞昱</t>
+          <t>中鋼</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.2056</v>
+        <v>0.2066</v>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>3533</t>
+          <t>2379</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>嘉澤</t>
+          <t>瑞昱</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.2051</v>
+        <v>0.2056</v>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3329,49 +3333,49 @@
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>1326</t>
+          <t>3533</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>台化</t>
+          <t>嘉澤</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.2011</v>
+        <v>0.2051</v>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>3034</t>
+          <t>1326</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>聯詠</t>
+          <t>台化</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.1996</v>
+        <v>0.2011</v>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
@@ -3381,26 +3385,26 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>6239</t>
+          <t>3034</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>力成</t>
+          <t>聯詠</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.1978</v>
+        <v>0.1996</v>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
@@ -3410,84 +3414,84 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>6239</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>亞德客-KY</t>
+          <t>力成</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.1925</v>
+        <v>0.1978</v>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>1519</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>華城</t>
+          <t>亞德客-KY</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.1898</v>
+        <v>0.1925</v>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>3044</t>
+          <t>1519</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>健鼎</t>
+          <t>華城</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.1883</v>
+        <v>0.1898</v>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
@@ -3503,49 +3507,49 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2207</t>
+          <t>3044</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>和泰車</t>
+          <t>健鼎</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.185</v>
+        <v>0.1883</v>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2356</t>
+          <t>2207</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>英業達</t>
+          <t>和泰車</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.1732</v>
+        <v>0.185</v>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
@@ -3555,89 +3559,89 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2376</t>
+          <t>2356</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>技嘉</t>
+          <t>英業達</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.1704</v>
+        <v>0.1732</v>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2801</t>
+          <t>2376</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>彰銀</t>
+          <t>技嘉</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.1638</v>
+        <v>0.1704</v>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>2801</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>和碩</t>
+          <t>彰銀</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.1632</v>
+        <v>0.1638</v>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3648,20 +3652,20 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>6415</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>和碩</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.1605</v>
+        <v>0.1632</v>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
@@ -3677,20 +3681,20 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2615</t>
+          <t>6415</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>萬海</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.1582</v>
+        <v>0.1605</v>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
@@ -3700,31 +3704,31 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2912</t>
+          <t>2615</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>統一超</t>
+          <t>萬海</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.153</v>
+        <v>0.1582</v>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3735,54 +3739,54 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2404</t>
+          <t>2912</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>漢唐</t>
+          <t>統一超</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0.1514</v>
+        <v>0.153</v>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>1802</t>
+          <t>2404</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>台玻</t>
+          <t>漢唐</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.1438</v>
+        <v>0.1514</v>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3793,170 +3797,170 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>3702</t>
+          <t>1802</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>大聯大</t>
+          <t>台玻</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.1357</v>
+        <v>0.1438</v>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2618</t>
+          <t>3702</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>長榮航</t>
+          <t>大聯大</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.1339</v>
+        <v>0.1357</v>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>6531</t>
+          <t>2618</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>長榮航</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.1331</v>
+        <v>0.1339</v>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>5876</t>
+          <t>6531</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>上海商銀</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.1329</v>
+        <v>0.1331</v>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2492</t>
+          <t>5876</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>華新科</t>
+          <t>上海商銀</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.1316</v>
+        <v>0.1329</v>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>6139</t>
+          <t>2492</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>亞翔</t>
+          <t>華新科</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.127</v>
+        <v>0.1316</v>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3967,45 +3971,45 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>5871</t>
+          <t>6139</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>中租-KY</t>
+          <t>亞翔</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0.1265</v>
+        <v>0.127</v>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2609</t>
+          <t>5871</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>陽明</t>
+          <t>中租-KY</t>
         </is>
       </c>
       <c r="D85" t="n">
@@ -4019,26 +4023,26 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>1101</t>
+          <t>2609</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>台泥</t>
+          <t>陽明</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.1262</v>
+        <v>0.1265</v>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
@@ -4048,26 +4052,26 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>1504</t>
+          <t>1101</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>東元</t>
+          <t>台泥</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.1226</v>
+        <v>0.1262</v>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
@@ -4077,26 +4081,26 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2409</t>
+          <t>1504</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>友達</t>
+          <t>東元</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.1194</v>
+        <v>0.1226</v>
       </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
@@ -4112,20 +4116,20 @@
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>1605</t>
+          <t>2409</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>華新</t>
+          <t>友達</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.1181</v>
+        <v>0.1194</v>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
@@ -4135,60 +4139,60 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>8210</t>
+          <t>1605</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>勤誠</t>
+          <t>華新</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.1176</v>
+        <v>0.1181</v>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2324</t>
+          <t>8210</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>仁寶</t>
+          <t>勤誠</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.1112</v>
+        <v>0.1176</v>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4199,25 +4203,25 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2834</t>
+          <t>2324</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>臺企銀</t>
+          <t>仁寶</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.1086</v>
+        <v>0.1112</v>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>金融🏦</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4228,25 +4232,25 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>6285</t>
+          <t>2834</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>啟碁</t>
+          <t>臺企銀</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.1061</v>
+        <v>0.1086</v>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>金融🏦</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4257,83 +4261,83 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2451</t>
+          <t>6285</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>創見</t>
+          <t>啟碁</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.1001</v>
+        <v>0.1061</v>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>🟡合理</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>6442</t>
+          <t>2451</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>創見</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.099</v>
+        <v>0.1001</v>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟡合理</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2347</t>
+          <t>6442</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>聯強</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.0985</v>
+        <v>0.099</v>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -4344,20 +4348,20 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2049</t>
+          <t>2347</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>上銀</t>
+          <t>聯強</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.0946</v>
+        <v>0.0985</v>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
@@ -4373,78 +4377,78 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>1402</t>
+          <t>2049</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>遠東新</t>
+          <t>上銀</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.0944</v>
+        <v>0.0946</v>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>3532</t>
+          <t>1402</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>台勝科</t>
+          <t>遠東新</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.0851</v>
+        <v>0.0944</v>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>1102</t>
+          <t>3532</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>亞泥</t>
+          <t>台勝科</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.0829</v>
+        <v>0.0851</v>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
@@ -4454,26 +4458,26 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🔴過熱</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>3706</t>
+          <t>1102</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>神達</t>
+          <t>亞泥</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.081</v>
+        <v>0.0829</v>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
@@ -4483,118 +4487,118 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2610</t>
+          <t>3706</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>華航</t>
+          <t>神達</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.0799</v>
+        <v>0.081</v>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>🟢便宜</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>2474</t>
+          <t>2610</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>可成</t>
+          <t>華航</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.0785</v>
+        <v>0.0799</v>
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>🟠偏貴</t>
+          <t>🟢便宜</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>1503</t>
+          <t>2474</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>士電</t>
+          <t>可成</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.0784</v>
+        <v>0.0785</v>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>🔴過熱</t>
+          <t>🟠偏貴</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>6196</t>
+          <t>1503</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>帆宣</t>
+          <t>士電</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.0774</v>
+        <v>0.0784</v>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -4605,28 +4609,57 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2812</t>
+          <t>6196</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>台中銀</t>
+          <t>帆宣</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.0764</v>
+        <v>0.0774</v>
       </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>🔴過熱</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>111</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2812</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>台中銀</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>0.0764</v>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
           <t>金融🏦</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr">
+      <c r="G107" t="inlineStr">
         <is>
           <t>🟠偏貴</t>
         </is>
@@ -10610,7 +10643,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6">

</xml_diff>